<commit_message>
Update Brine Concentrator ZO (#1802)
* add validity range and add costing tests

* crystallizer ZO as separate model; correct error in capex calculation

* fix tests

* black

* automate zo docs and add crystallizer

* update .xlsx to use crystallizer for name

* re-run autodocs for zo models

* rename crystallizer zo test file

* use q_out

* docs untis fix 1

Co-authored-by: jakechurchi <jake.churchill@nlr.gov>

* docs units fix 2

Co-authored-by: jakechurchi <jake.churchill@nlr.gov>

* docs units fix 3

Co-authored-by: jakechurchi <jake.churchill@nlr.gov>

* yaml changes from comments

* fix crystallizer test

* remove unused factor

* clean up

* authorship

* fix docx merge conflicts

* classmethod

* classmethod

---------

Co-authored-by: jakechurchi <jake.churchill@nlr.gov>
</commit_message>
<xml_diff>
--- a/docs/technical_reference/unit_models/zero_order_unit_models/WT3_unit_classification_for_doc.xlsx
+++ b/docs/technical_reference/unit_models/zero_order_unit_models/WT3_unit_classification_for_doc.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10531"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C43B9EE-BEE0-BB49-8E61-51C4620CFE4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7C1B3F5-E496-E348-B5C9-5A5374BB4600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10580" yWindow="2740" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$92</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="993" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="515">
   <si>
     <t>Name</t>
   </si>
@@ -1565,6 +1565,18 @@
   </si>
   <si>
     <t>cost_electrocoagulation</t>
+  </si>
+  <si>
+    <t>crystallizer_zo</t>
+  </si>
+  <si>
+    <t>CrystallizerZO</t>
+  </si>
+  <si>
+    <t>cost_crystallizer</t>
+  </si>
+  <si>
+    <t>crystallizer</t>
   </si>
 </sst>
 </file>
@@ -1938,7 +1950,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J91"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33.5" customWidth="1"/>
@@ -2011,11 +2023,11 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I2" t="str">
-        <f t="shared" ref="I2:I38" si="1">IF(E2="SIDO","single-input, double-output",IF(E2="SISO","single-input, single-output",IF(E2="PT","pass-through",IF(E2="DISO","double-input, single-output",IF(E2="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
+        <f t="shared" ref="I2:I39" si="1">IF(E2="SIDO","single-input, double-output",IF(E2="SISO","single-input, single-output",IF(E2="PT","pass-through",IF(E2="DISO","double-input, single-output",IF(E2="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
         <v>single-input, double-output</v>
       </c>
       <c r="J2" t="str">
-        <f t="shared" ref="J2:J38" si="2">IF(E2="SIDO","sido_methods",IF(E2="SISO","siso_methods",IF(E2="PT","pt_methods",IF(E2="DISO","diso_methods",IF(E2="SIDO reactive","sidor_methods","")))))</f>
+        <f t="shared" ref="J2:J39" si="2">IF(E2="SIDO","sido_methods",IF(E2="SISO","siso_methods",IF(E2="PT","pt_methods",IF(E2="DISO","diso_methods",IF(E2="SIDO reactive","sidor_methods","")))))</f>
         <v>sido_methods</v>
       </c>
     </row>
@@ -2883,254 +2895,254 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>514</v>
+      </c>
+      <c r="B28" t="s">
+        <v>511</v>
+      </c>
+      <c r="C28" t="s">
+        <v>512</v>
+      </c>
+      <c r="D28" t="s">
+        <v>30</v>
+      </c>
+      <c r="E28" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" t="b">
+        <v>0</v>
+      </c>
+      <c r="G28" t="s">
+        <v>31</v>
+      </c>
+      <c r="H28" t="s">
+        <v>513</v>
+      </c>
+      <c r="I28" t="str">
+        <f t="shared" ref="I28" si="3">IF(E28="SIDO","single-input, double-output",IF(E28="SISO","single-input, single-output",IF(E28="PT","pass-through",IF(E28="DISO","double-input, single-output",IF(E28="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
+        <v>single-input, double-output</v>
+      </c>
+      <c r="J28" t="str">
+        <f t="shared" ref="J28" si="4">IF(E28="SIDO","sido_methods",IF(E28="SISO","siso_methods",IF(E28="PT","pt_methods",IF(E28="DISO","diso_methods",IF(E28="SIDO reactive","sidor_methods","")))))</f>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
         <v>66</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>67</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C29" t="s">
         <v>390</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D29" t="s">
         <v>10</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E29" t="s">
         <v>26</v>
       </c>
-      <c r="F28" t="b">
+      <c r="F29" t="b">
         <v>1</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G29" t="s">
         <v>12</v>
       </c>
-      <c r="H28" t="str">
-        <f>IF(D28="basic","cost_power_law_flow")</f>
+      <c r="H29" t="str">
+        <f>IF(D29="basic","cost_power_law_flow")</f>
         <v>cost_power_law_flow</v>
       </c>
-      <c r="I28" t="str">
+      <c r="I29" t="str">
         <f t="shared" si="1"/>
         <v>single-input, single-output</v>
       </c>
-      <c r="J28" t="str">
+      <c r="J29" t="str">
         <f t="shared" si="2"/>
         <v>siso_methods</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
         <v>68</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B30" t="s">
         <v>69</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C30" t="s">
         <v>379</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D30" t="s">
         <v>30</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E30" t="s">
         <v>27</v>
       </c>
-      <c r="F29" t="b">
+      <c r="F30" t="b">
         <v>1</v>
       </c>
-      <c r="G29" t="s">
+      <c r="G30" t="s">
         <v>21</v>
       </c>
-      <c r="H29" t="s">
+      <c r="H30" t="s">
         <v>70</v>
       </c>
-      <c r="I29" t="str">
+      <c r="I30" t="str">
         <f t="shared" si="1"/>
         <v>pass-through</v>
       </c>
-      <c r="J29" t="str">
+      <c r="J30" t="str">
         <f t="shared" si="2"/>
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
         <v>71</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B31" t="s">
         <v>72</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C31" t="s">
         <v>391</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D31" t="s">
         <v>10</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E31" t="s">
         <v>11</v>
       </c>
-      <c r="F30" t="b">
+      <c r="F31" t="b">
         <v>1</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G31" t="s">
         <v>12</v>
       </c>
-      <c r="H30" t="str">
-        <f>IF(D30="basic","cost_power_law_flow")</f>
+      <c r="H31" t="str">
+        <f>IF(D31="basic","cost_power_law_flow")</f>
         <v>cost_power_law_flow</v>
       </c>
-      <c r="I30" t="str">
+      <c r="I31" t="str">
         <f t="shared" si="1"/>
         <v>single-input, double-output</v>
       </c>
-      <c r="J30" t="str">
+      <c r="J31" t="str">
         <f t="shared" si="2"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
         <v>73</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B32" t="s">
         <v>74</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C32" t="s">
         <v>380</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D32" t="s">
         <v>57</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E32" t="s">
         <v>18</v>
       </c>
-      <c r="F31" t="b">
+      <c r="F32" t="b">
         <v>1</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G32" t="s">
         <v>12</v>
       </c>
-      <c r="H31" t="s">
+      <c r="H32" t="s">
         <v>75</v>
       </c>
-      <c r="I31" t="str">
+      <c r="I32" t="str">
         <f t="shared" si="1"/>
         <v>reactive single-inlet, double-outlet</v>
       </c>
-      <c r="J31" t="str">
+      <c r="J32" t="str">
         <f t="shared" si="2"/>
         <v>sidor_methods</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
         <v>76</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B33" t="s">
         <v>77</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C33" t="s">
         <v>429</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D33" t="s">
         <v>10</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E33" t="s">
         <v>11</v>
       </c>
-      <c r="F32" t="b">
+      <c r="F33" t="b">
         <v>1</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G33" t="s">
         <v>12</v>
       </c>
-      <c r="H32" t="str">
-        <f>IF(D32="basic","cost_power_law_flow")</f>
+      <c r="H33" t="str">
+        <f>IF(D33="basic","cost_power_law_flow")</f>
         <v>cost_power_law_flow</v>
       </c>
-      <c r="I32" t="str">
+      <c r="I33" t="str">
         <f t="shared" si="1"/>
         <v>single-input, double-output</v>
       </c>
-      <c r="J32" t="str">
+      <c r="J33" t="str">
         <f t="shared" si="2"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
         <v>78</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>79</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C34" t="s">
         <v>394</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D34" t="s">
         <v>30</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E34" t="s">
         <v>18</v>
       </c>
-      <c r="F33" t="b">
+      <c r="F34" t="b">
         <v>0</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G34" t="s">
         <v>31</v>
       </c>
-      <c r="H33" t="s">
+      <c r="H34" t="s">
         <v>80</v>
       </c>
-      <c r="I33" t="str">
+      <c r="I34" t="str">
         <f t="shared" si="1"/>
         <v>reactive single-inlet, double-outlet</v>
       </c>
-      <c r="J33" t="str">
+      <c r="J34" t="str">
         <f t="shared" si="2"/>
         <v>sidor_methods</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>507</v>
-      </c>
-      <c r="B34" t="s">
-        <v>508</v>
-      </c>
-      <c r="C34" t="s">
-        <v>509</v>
-      </c>
-      <c r="D34" t="s">
-        <v>30</v>
-      </c>
-      <c r="E34" t="s">
-        <v>11</v>
-      </c>
-      <c r="F34" t="b">
-        <v>0</v>
-      </c>
-      <c r="G34" t="s">
-        <v>31</v>
-      </c>
-      <c r="H34" t="s">
-        <v>510</v>
-      </c>
-      <c r="I34" t="str">
-        <f t="shared" si="1"/>
-        <v>single-input, double-output</v>
-      </c>
-      <c r="J34" t="str">
-        <f t="shared" si="2"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>81</v>
+        <v>507</v>
       </c>
       <c r="B35" t="s">
-        <v>82</v>
+        <v>508</v>
       </c>
       <c r="C35" t="s">
-        <v>381</v>
+        <v>509</v>
       </c>
       <c r="D35" t="s">
         <v>30</v>
@@ -3145,7 +3157,7 @@
         <v>31</v>
       </c>
       <c r="H35" t="s">
-        <v>65</v>
+        <v>510</v>
       </c>
       <c r="I35" t="str">
         <f t="shared" si="1"/>
@@ -3158,54 +3170,53 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B36" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C36" t="s">
-        <v>395</v>
+        <v>381</v>
       </c>
       <c r="D36" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E36" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G36" t="s">
-        <v>12</v>
-      </c>
-      <c r="H36" t="str">
-        <f>IF(D36="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>31</v>
+      </c>
+      <c r="H36" t="s">
+        <v>65</v>
       </c>
       <c r="I36" t="str">
         <f t="shared" si="1"/>
-        <v>pass-through</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J36" t="str">
         <f t="shared" si="2"/>
-        <v>pt_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B37" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C37" t="s">
-        <v>436</v>
+        <v>395</v>
       </c>
       <c r="D37" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E37" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F37" t="b">
         <v>1</v>
@@ -3213,33 +3224,34 @@
       <c r="G37" t="s">
         <v>12</v>
       </c>
-      <c r="H37" t="s">
-        <v>87</v>
+      <c r="H37" t="str">
+        <f>IF(D37="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I37" t="str">
         <f t="shared" si="1"/>
-        <v>single-input, double-output</v>
+        <v>pass-through</v>
       </c>
       <c r="J37" t="str">
         <f t="shared" si="2"/>
-        <v>sido_methods</v>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B38" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C38" t="s">
-        <v>392</v>
+        <v>436</v>
       </c>
       <c r="D38" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E38" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F38" t="b">
         <v>1</v>
@@ -3247,163 +3259,163 @@
       <c r="G38" t="s">
         <v>12</v>
       </c>
-      <c r="H38" t="str">
-        <f>IF(D38="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H38" t="s">
+        <v>87</v>
       </c>
       <c r="I38" t="str">
         <f t="shared" si="1"/>
-        <v>pass-through</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J38" t="str">
         <f t="shared" si="2"/>
-        <v>pt_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B39" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C39" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D39" t="s">
-        <v>92</v>
+        <v>10</v>
       </c>
       <c r="E39" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="F39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G39" t="s">
-        <v>58</v>
-      </c>
-      <c r="H39" t="b">
+        <v>12</v>
+      </c>
+      <c r="H39" t="str">
         <f>IF(D39="basic","cost_power_law_flow")</f>
-        <v>0</v>
-      </c>
-      <c r="I39" t="s">
-        <v>93</v>
-      </c>
-      <c r="J39" t="s">
-        <v>93</v>
+        <v>cost_power_law_flow</v>
+      </c>
+      <c r="I39" t="str">
+        <f t="shared" si="1"/>
+        <v>pass-through</v>
+      </c>
+      <c r="J39" t="str">
+        <f t="shared" si="2"/>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B40" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C40" t="s">
-        <v>437</v>
+        <v>393</v>
       </c>
       <c r="D40" t="s">
-        <v>30</v>
+        <v>92</v>
       </c>
       <c r="E40" t="s">
-        <v>11</v>
+        <v>58</v>
       </c>
       <c r="F40" t="b">
         <v>0</v>
       </c>
       <c r="G40" t="s">
-        <v>31</v>
-      </c>
-      <c r="H40" t="s">
-        <v>96</v>
-      </c>
-      <c r="I40" t="str">
-        <f t="shared" ref="I40:I45" si="3">IF(E40="SIDO","single-input, double-output",IF(E40="SISO","single-input, single-output",IF(E40="PT","pass-through",IF(E40="DISO","double-input, single-output",IF(E40="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
-        <v>single-input, double-output</v>
-      </c>
-      <c r="J40" t="str">
-        <f t="shared" ref="J40:J45" si="4">IF(E40="SIDO","sido_methods",IF(E40="SISO","siso_methods",IF(E40="PT","pt_methods",IF(E40="DISO","diso_methods",IF(E40="SIDO reactive","sidor_methods","")))))</f>
-        <v>sido_methods</v>
+        <v>58</v>
+      </c>
+      <c r="H40" t="b">
+        <f>IF(D40="basic","cost_power_law_flow")</f>
+        <v>0</v>
+      </c>
+      <c r="I40" t="s">
+        <v>93</v>
+      </c>
+      <c r="J40" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B41" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C41" t="s">
-        <v>422</v>
+        <v>437</v>
       </c>
       <c r="D41" t="s">
         <v>30</v>
       </c>
       <c r="E41" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="H41" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I41" t="str">
-        <f t="shared" si="3"/>
-        <v>single-input, single-output</v>
+        <f t="shared" ref="I41:I46" si="5">IF(E41="SIDO","single-input, double-output",IF(E41="SISO","single-input, single-output",IF(E41="PT","pass-through",IF(E41="DISO","double-input, single-output",IF(E41="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
+        <v>single-input, double-output</v>
       </c>
       <c r="J41" t="str">
-        <f t="shared" si="4"/>
-        <v>siso_methods</v>
+        <f t="shared" ref="J41:J46" si="6">IF(E41="SIDO","sido_methods",IF(E41="SISO","siso_methods",IF(E41="PT","pt_methods",IF(E41="DISO","diso_methods",IF(E41="SIDO reactive","sidor_methods","")))))</f>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B42" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C42" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
       <c r="D42" t="s">
         <v>30</v>
       </c>
       <c r="E42" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G42" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H42" t="s">
-        <v>506</v>
+        <v>99</v>
       </c>
       <c r="I42" t="str">
-        <f t="shared" si="3"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="5"/>
+        <v>single-input, single-output</v>
       </c>
       <c r="J42" t="str">
-        <f t="shared" si="4"/>
-        <v>sido_methods</v>
+        <f t="shared" si="6"/>
+        <v>siso_methods</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B43" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C43" t="s">
-        <v>450</v>
+        <v>428</v>
       </c>
       <c r="D43" t="s">
         <v>30</v>
@@ -3412,69 +3424,69 @@
         <v>11</v>
       </c>
       <c r="F43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G43" t="s">
-        <v>21</v>
-      </c>
-      <c r="H43" t="b">
-        <v>0</v>
+        <v>31</v>
+      </c>
+      <c r="H43" t="s">
+        <v>506</v>
       </c>
       <c r="I43" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J43" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>474</v>
+        <v>102</v>
       </c>
       <c r="B44" t="s">
-        <v>473</v>
+        <v>103</v>
       </c>
       <c r="C44" t="s">
-        <v>475</v>
+        <v>450</v>
       </c>
       <c r="D44" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E44" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F44" t="b">
         <v>1</v>
       </c>
       <c r="G44" t="s">
-        <v>12</v>
-      </c>
-      <c r="H44" t="s">
-        <v>476</v>
+        <v>21</v>
+      </c>
+      <c r="H44" t="b">
+        <v>0</v>
       </c>
       <c r="I44" t="str">
-        <f t="shared" si="3"/>
-        <v>reactive single-inlet, double-outlet</v>
+        <f t="shared" si="5"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J44" t="str">
-        <f t="shared" si="4"/>
-        <v>sidor_methods</v>
+        <f t="shared" si="6"/>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="B45" t="s">
-        <v>455</v>
+        <v>473</v>
       </c>
       <c r="C45" t="s">
-        <v>451</v>
+        <v>475</v>
       </c>
       <c r="D45" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E45" t="s">
         <v>18</v>
@@ -3483,64 +3495,63 @@
         <v>1</v>
       </c>
       <c r="G45" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H45" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="I45" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J45" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>sidor_methods</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>104</v>
+        <v>477</v>
       </c>
       <c r="B46" t="s">
-        <v>105</v>
+        <v>455</v>
       </c>
       <c r="C46" t="s">
-        <v>441</v>
+        <v>451</v>
       </c>
       <c r="D46" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E46" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="F46" t="b">
         <v>1</v>
       </c>
       <c r="G46" t="s">
-        <v>12</v>
-      </c>
-      <c r="H46" t="str">
-        <f>IF(D46="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>31</v>
+      </c>
+      <c r="H46" t="s">
+        <v>478</v>
       </c>
       <c r="I46" t="str">
-        <f t="shared" ref="I46:I91" si="5">IF(E46="SIDO","single-input, double-output",IF(E46="SISO","single-input, single-output",IF(E46="PT","pass-through",IF(E46="DISO","double-input, single-output",IF(E46="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
-        <v>pass-through</v>
+        <f t="shared" si="5"/>
+        <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J46" t="str">
-        <f t="shared" ref="J46:J91" si="6">IF(E46="SIDO","sido_methods",IF(E46="SISO","siso_methods",IF(E46="PT","pt_methods",IF(E46="DISO","diso_methods",IF(E46="SIDO reactive","sidor_methods","")))))</f>
-        <v>pt_methods</v>
+        <f t="shared" si="6"/>
+        <v>sidor_methods</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B47" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C47" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D47" t="s">
         <v>10</v>
@@ -3559,57 +3570,58 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I47" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="I47:I92" si="7">IF(E47="SIDO","single-input, double-output",IF(E47="SISO","single-input, single-output",IF(E47="PT","pass-through",IF(E47="DISO","double-input, single-output",IF(E47="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
         <v>pass-through</v>
       </c>
       <c r="J47" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="J47:J92" si="8">IF(E47="SIDO","sido_methods",IF(E47="SISO","siso_methods",IF(E47="PT","pt_methods",IF(E47="DISO","diso_methods",IF(E47="SIDO reactive","sidor_methods","")))))</f>
         <v>pt_methods</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B48" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C48" t="s">
-        <v>426</v>
+        <v>440</v>
       </c>
       <c r="D48" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E48" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F48" t="b">
         <v>1</v>
       </c>
       <c r="G48" t="s">
-        <v>21</v>
-      </c>
-      <c r="H48" t="s">
-        <v>110</v>
+        <v>12</v>
+      </c>
+      <c r="H48" t="str">
+        <f>IF(D48="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I48" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>pass-through</v>
       </c>
       <c r="J48" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
+        <f t="shared" si="8"/>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B49" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C49" t="s">
-        <v>396</v>
+        <v>426</v>
       </c>
       <c r="D49" t="s">
         <v>30</v>
@@ -3618,72 +3630,72 @@
         <v>11</v>
       </c>
       <c r="F49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G49" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H49" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I49" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J49" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B50" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C50" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="D50" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E50" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G50" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="H50" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="I50" t="str">
-        <f t="shared" si="5"/>
-        <v>pass-through</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J50" t="str">
-        <f t="shared" si="6"/>
-        <v>pt_methods</v>
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B51" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C51" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="D51" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E51" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F51" t="b">
         <v>1</v>
@@ -3692,26 +3704,26 @@
         <v>12</v>
       </c>
       <c r="H51" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I51" t="str">
-        <f t="shared" si="5"/>
-        <v>reactive single-inlet, double-outlet</v>
+        <f t="shared" si="7"/>
+        <v>pass-through</v>
       </c>
       <c r="J51" t="str">
-        <f t="shared" si="6"/>
-        <v>sidor_methods</v>
+        <f t="shared" si="8"/>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>479</v>
+        <v>117</v>
       </c>
       <c r="B52" t="s">
-        <v>480</v>
+        <v>118</v>
       </c>
       <c r="C52" t="s">
-        <v>481</v>
+        <v>399</v>
       </c>
       <c r="D52" t="s">
         <v>30</v>
@@ -3726,32 +3738,32 @@
         <v>12</v>
       </c>
       <c r="H52" t="s">
-        <v>482</v>
+        <v>119</v>
       </c>
       <c r="I52" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J52" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sidor_methods</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>120</v>
+        <v>479</v>
       </c>
       <c r="B53" t="s">
-        <v>121</v>
+        <v>480</v>
       </c>
       <c r="C53" t="s">
-        <v>400</v>
+        <v>481</v>
       </c>
       <c r="D53" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E53" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F53" t="b">
         <v>1</v>
@@ -3759,28 +3771,27 @@
       <c r="G53" t="s">
         <v>12</v>
       </c>
-      <c r="H53" t="str">
-        <f>IF(D53="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H53" t="s">
+        <v>482</v>
       </c>
       <c r="I53" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J53" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
+        <f t="shared" si="8"/>
+        <v>sidor_methods</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B54" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C54" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D54" t="s">
         <v>10</v>
@@ -3799,26 +3810,26 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I54" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J54" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>483</v>
+        <v>122</v>
       </c>
       <c r="B55" t="s">
-        <v>484</v>
+        <v>123</v>
       </c>
       <c r="C55" t="s">
-        <v>485</v>
+        <v>401</v>
       </c>
       <c r="D55" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E55" t="s">
         <v>11</v>
@@ -3829,61 +3840,62 @@
       <c r="G55" t="s">
         <v>12</v>
       </c>
-      <c r="H55" t="s">
-        <v>486</v>
+      <c r="H55" t="str">
+        <f>IF(D55="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I55" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J55" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>124</v>
+        <v>483</v>
       </c>
       <c r="B56" t="s">
-        <v>125</v>
+        <v>484</v>
       </c>
       <c r="C56" t="s">
-        <v>385</v>
+        <v>485</v>
       </c>
       <c r="D56" t="s">
         <v>30</v>
       </c>
       <c r="E56" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F56" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G56" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H56" t="s">
-        <v>126</v>
+        <v>486</v>
       </c>
       <c r="I56" t="str">
-        <f t="shared" si="5"/>
-        <v>reactive single-inlet, double-outlet</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J56" t="str">
-        <f t="shared" si="6"/>
-        <v>sidor_methods</v>
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>487</v>
+        <v>124</v>
       </c>
       <c r="B57" t="s">
-        <v>488</v>
+        <v>125</v>
       </c>
       <c r="C57" t="s">
-        <v>489</v>
+        <v>385</v>
       </c>
       <c r="D57" t="s">
         <v>30</v>
@@ -3892,38 +3904,38 @@
         <v>18</v>
       </c>
       <c r="F57" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G57" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="H57" t="s">
-        <v>490</v>
+        <v>126</v>
       </c>
       <c r="I57" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J57" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sidor_methods</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>127</v>
+        <v>487</v>
       </c>
       <c r="B58" t="s">
-        <v>128</v>
+        <v>488</v>
       </c>
       <c r="C58" t="s">
-        <v>402</v>
+        <v>489</v>
       </c>
       <c r="D58" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E58" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F58" t="b">
         <v>1</v>
@@ -3931,62 +3943,62 @@
       <c r="G58" t="s">
         <v>12</v>
       </c>
-      <c r="H58" t="str">
-        <f>IF(D58="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H58" t="s">
+        <v>490</v>
       </c>
       <c r="I58" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J58" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
+        <f t="shared" si="8"/>
+        <v>sidor_methods</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B59" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C59" t="s">
-        <v>423</v>
+        <v>402</v>
       </c>
       <c r="D59" t="s">
         <v>10</v>
       </c>
       <c r="E59" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F59" t="b">
         <v>1</v>
       </c>
       <c r="G59" t="s">
-        <v>21</v>
-      </c>
-      <c r="H59" t="s">
-        <v>65</v>
+        <v>12</v>
+      </c>
+      <c r="H59" t="str">
+        <f>IF(D59="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I59" t="str">
-        <f t="shared" si="5"/>
-        <v>pass-through</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J59" t="str">
-        <f t="shared" si="6"/>
-        <v>pt_methods</v>
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B60" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C60" t="s">
-        <v>404</v>
+        <v>423</v>
       </c>
       <c r="D60" t="s">
         <v>10</v>
@@ -3998,70 +4010,70 @@
         <v>1</v>
       </c>
       <c r="G60" t="s">
-        <v>12</v>
-      </c>
-      <c r="H60" t="str">
-        <f>IF(D60="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>21</v>
+      </c>
+      <c r="H60" t="s">
+        <v>65</v>
       </c>
       <c r="I60" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
       <c r="J60" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B61" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C61" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="D61" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E61" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G61" t="s">
-        <v>31</v>
-      </c>
-      <c r="H61" t="s">
-        <v>136</v>
+        <v>12</v>
+      </c>
+      <c r="H61" t="str">
+        <f>IF(D61="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I61" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>pass-through</v>
       </c>
       <c r="J61" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
+        <f t="shared" si="8"/>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B62" t="s">
-        <v>369</v>
+        <v>135</v>
       </c>
       <c r="C62" t="s">
-        <v>425</v>
+        <v>405</v>
       </c>
       <c r="D62" t="s">
         <v>30</v>
       </c>
       <c r="E62" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F62" t="b">
         <v>0</v>
@@ -4070,26 +4082,26 @@
         <v>31</v>
       </c>
       <c r="H62" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I62" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, single-output</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J62" t="str">
-        <f t="shared" si="6"/>
-        <v>siso_methods</v>
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B63" t="s">
-        <v>140</v>
+        <v>369</v>
       </c>
       <c r="C63" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D63" t="s">
         <v>30</v>
@@ -4104,204 +4116,203 @@
         <v>31</v>
       </c>
       <c r="H63" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="I63" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, single-output</v>
       </c>
       <c r="J63" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>siso_methods</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>491</v>
+        <v>139</v>
       </c>
       <c r="B64" t="s">
-        <v>492</v>
+        <v>140</v>
       </c>
       <c r="C64" t="s">
-        <v>493</v>
+        <v>424</v>
       </c>
       <c r="D64" t="s">
         <v>30</v>
       </c>
       <c r="E64" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F64" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G64" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="H64" t="s">
-        <v>494</v>
+        <v>141</v>
       </c>
       <c r="I64" t="str">
-        <f t="shared" si="5"/>
-        <v>reactive single-inlet, double-outlet</v>
+        <f t="shared" si="7"/>
+        <v>single-input, single-output</v>
       </c>
       <c r="J64" t="str">
-        <f t="shared" si="6"/>
-        <v>sidor_methods</v>
+        <f t="shared" si="8"/>
+        <v>siso_methods</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>142</v>
+        <v>491</v>
       </c>
       <c r="B65" t="s">
-        <v>143</v>
+        <v>492</v>
       </c>
       <c r="C65" t="s">
-        <v>443</v>
+        <v>493</v>
       </c>
       <c r="D65" t="s">
         <v>30</v>
       </c>
       <c r="E65" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G65" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H65" t="s">
-        <v>144</v>
+        <v>494</v>
       </c>
       <c r="I65" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J65" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
+        <f t="shared" si="8"/>
+        <v>sidor_methods</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B66" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C66" t="s">
-        <v>407</v>
+        <v>443</v>
       </c>
       <c r="D66" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E66" t="s">
         <v>11</v>
       </c>
       <c r="F66" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G66" t="s">
-        <v>12</v>
-      </c>
-      <c r="H66" t="str">
-        <f>IF(D66="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>31</v>
+      </c>
+      <c r="H66" t="s">
+        <v>144</v>
       </c>
       <c r="I66" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J66" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B67" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C67" t="s">
-        <v>398</v>
+        <v>407</v>
       </c>
       <c r="D67" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E67" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G67" t="s">
-        <v>31</v>
-      </c>
-      <c r="H67" t="s">
-        <v>149</v>
+        <v>12</v>
+      </c>
+      <c r="H67" t="str">
+        <f>IF(D67="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I67" t="str">
-        <f t="shared" si="5"/>
-        <v>pass-through</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J67" t="str">
-        <f t="shared" si="6"/>
-        <v>pt_methods</v>
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B68" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C68" t="s">
-        <v>408</v>
+        <v>398</v>
       </c>
       <c r="D68" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E68" t="s">
         <v>27</v>
       </c>
       <c r="F68" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G68" t="s">
-        <v>12</v>
-      </c>
-      <c r="H68" t="str">
-        <f>IF(D68="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>31</v>
+      </c>
+      <c r="H68" t="s">
+        <v>149</v>
       </c>
       <c r="I68" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
       <c r="J68" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B69" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C69" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="D69" t="s">
         <v>10</v>
       </c>
       <c r="E69" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F69" t="b">
         <v>1</v>
@@ -4314,26 +4325,26 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I69" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>pass-through</v>
       </c>
       <c r="J69" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
+        <f t="shared" si="8"/>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B70" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C70" t="s">
-        <v>447</v>
+        <v>409</v>
       </c>
       <c r="D70" t="s">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="E70" t="s">
         <v>11</v>
@@ -4344,30 +4355,31 @@
       <c r="G70" t="s">
         <v>12</v>
       </c>
-      <c r="H70" t="s">
-        <v>65</v>
+      <c r="H70" t="str">
+        <f>IF(D70="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I70" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J70" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B71" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C71" t="s">
-        <v>410</v>
+        <v>447</v>
       </c>
       <c r="D71" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="E71" t="s">
         <v>11</v>
@@ -4379,29 +4391,29 @@
         <v>12</v>
       </c>
       <c r="H71" t="s">
-        <v>158</v>
+        <v>65</v>
       </c>
       <c r="I71" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J71" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B72" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C72" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="D72" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E72" t="s">
         <v>11</v>
@@ -4412,28 +4424,27 @@
       <c r="G72" t="s">
         <v>12</v>
       </c>
-      <c r="H72" t="str">
-        <f>IF(D72="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H72" t="s">
+        <v>158</v>
       </c>
       <c r="I72" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J72" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B73" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C73" t="s">
-        <v>435</v>
+        <v>411</v>
       </c>
       <c r="D73" t="s">
         <v>10</v>
@@ -4452,29 +4463,29 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I73" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J73" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B74" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C74" t="s">
-        <v>412</v>
+        <v>435</v>
       </c>
       <c r="D74" t="s">
         <v>10</v>
       </c>
       <c r="E74" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F74" t="b">
         <v>1</v>
@@ -4487,23 +4498,23 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I74" t="str">
-        <f t="shared" si="5"/>
-        <v>pass-through</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J74" t="str">
-        <f t="shared" si="6"/>
-        <v>pt_methods</v>
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B75" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C75" t="s">
-        <v>433</v>
+        <v>412</v>
       </c>
       <c r="D75" t="s">
         <v>10</v>
@@ -4522,26 +4533,26 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I75" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
       <c r="J75" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B76" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C76" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="D76" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E76" t="s">
         <v>27</v>
@@ -4552,30 +4563,31 @@
       <c r="G76" t="s">
         <v>12</v>
       </c>
-      <c r="H76" t="s">
-        <v>169</v>
+      <c r="H76" t="str">
+        <f>IF(D76="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I76" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
       <c r="J76" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>495</v>
+        <v>167</v>
       </c>
       <c r="B77" t="s">
-        <v>496</v>
+        <v>168</v>
       </c>
       <c r="C77" t="s">
-        <v>497</v>
+        <v>430</v>
       </c>
       <c r="D77" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E77" t="s">
         <v>27</v>
@@ -4587,32 +4599,32 @@
         <v>12</v>
       </c>
       <c r="H77" t="s">
-        <v>498</v>
+        <v>169</v>
       </c>
       <c r="I77" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
       <c r="J77" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="B78" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="C78" t="s">
-        <v>501</v>
+        <v>497</v>
       </c>
       <c r="D78" t="s">
         <v>10</v>
       </c>
       <c r="E78" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F78" t="b">
         <v>1</v>
@@ -4621,97 +4633,97 @@
         <v>12</v>
       </c>
       <c r="H78" t="s">
-        <v>502</v>
+        <v>498</v>
       </c>
       <c r="I78" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>pass-through</v>
       </c>
       <c r="J78" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
+        <f t="shared" si="8"/>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="B79" t="s">
-        <v>456</v>
+        <v>500</v>
       </c>
       <c r="C79" t="s">
-        <v>452</v>
+        <v>501</v>
       </c>
       <c r="D79" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E79" t="s">
         <v>11</v>
       </c>
       <c r="F79" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G79" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H79" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="I79" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J79" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>170</v>
+        <v>503</v>
       </c>
       <c r="B80" t="s">
-        <v>171</v>
+        <v>456</v>
       </c>
       <c r="C80" t="s">
-        <v>442</v>
+        <v>452</v>
       </c>
       <c r="D80" t="s">
         <v>30</v>
       </c>
       <c r="E80" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F80" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G80" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="H80" t="s">
-        <v>172</v>
+        <v>504</v>
       </c>
       <c r="I80" t="str">
-        <f t="shared" si="5"/>
-        <v>pass-through</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J80" t="str">
-        <f t="shared" si="6"/>
-        <v>pt_methods</v>
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B81" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="C81" t="s">
-        <v>431</v>
+        <v>442</v>
       </c>
       <c r="D81" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E81" t="s">
         <v>27</v>
@@ -4722,28 +4734,27 @@
       <c r="G81" t="s">
         <v>21</v>
       </c>
-      <c r="H81" t="str">
-        <f>IF(D81="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H81" t="s">
+        <v>172</v>
       </c>
       <c r="I81" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
       <c r="J81" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B82" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C82" t="s">
-        <v>413</v>
+        <v>431</v>
       </c>
       <c r="D82" t="s">
         <v>10</v>
@@ -4755,36 +4766,36 @@
         <v>1</v>
       </c>
       <c r="G82" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="H82" t="str">
         <f>IF(D82="basic","cost_power_law_flow")</f>
         <v>cost_power_law_flow</v>
       </c>
       <c r="I82" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
       <c r="J82" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B83" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C83" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D83" t="s">
         <v>10</v>
       </c>
       <c r="E83" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F83" t="b">
         <v>1</v>
@@ -4797,23 +4808,23 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I83" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>pass-through</v>
       </c>
       <c r="J83" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
+        <f t="shared" si="8"/>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B84" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C84" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D84" t="s">
         <v>10</v>
@@ -4832,29 +4843,29 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I84" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J84" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B85" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C85" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D85" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E85" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F85" t="b">
         <v>1</v>
@@ -4862,27 +4873,28 @@
       <c r="G85" t="s">
         <v>12</v>
       </c>
-      <c r="H85" t="s">
-        <v>183</v>
+      <c r="H85" t="str">
+        <f>IF(D85="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I85" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, single-output</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J85" t="str">
-        <f t="shared" si="6"/>
-        <v>siso_methods</v>
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B86" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C86" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D86" t="s">
         <v>30</v>
@@ -4897,32 +4909,32 @@
         <v>12</v>
       </c>
       <c r="H86" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="I86" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, single-output</v>
       </c>
       <c r="J86" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>siso_methods</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B87" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C87" t="s">
-        <v>453</v>
+        <v>417</v>
       </c>
       <c r="D87" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="E87" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F87" t="b">
         <v>1</v>
@@ -4931,29 +4943,29 @@
         <v>12</v>
       </c>
       <c r="H87" t="s">
-        <v>460</v>
+        <v>186</v>
       </c>
       <c r="I87" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>single-input, single-output</v>
       </c>
       <c r="J87" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
+        <f t="shared" si="8"/>
+        <v>siso_methods</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B88" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C88" t="s">
-        <v>420</v>
+        <v>453</v>
       </c>
       <c r="D88" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="E88" t="s">
         <v>11</v>
@@ -4964,28 +4976,27 @@
       <c r="G88" t="s">
         <v>12</v>
       </c>
-      <c r="H88" t="str">
-        <f>IF(D88="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H88" t="s">
+        <v>460</v>
       </c>
       <c r="I88" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J88" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B89" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C89" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D89" t="s">
         <v>10</v>
@@ -5004,57 +5015,58 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I89" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J89" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B90" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C90" t="s">
-        <v>438</v>
+        <v>419</v>
       </c>
       <c r="D90" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E90" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F90" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G90" t="s">
-        <v>31</v>
-      </c>
-      <c r="H90" t="s">
-        <v>65</v>
+        <v>12</v>
+      </c>
+      <c r="H90" t="str">
+        <f>IF(D90="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I90" t="str">
-        <f t="shared" si="5"/>
-        <v>pass-through</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J90" t="str">
-        <f t="shared" si="6"/>
-        <v>pt_methods</v>
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B91" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C91" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="D91" t="s">
         <v>30</v>
@@ -5063,26 +5075,60 @@
         <v>27</v>
       </c>
       <c r="F91" t="b">
+        <v>0</v>
+      </c>
+      <c r="G91" t="s">
+        <v>31</v>
+      </c>
+      <c r="H91" t="s">
+        <v>65</v>
+      </c>
+      <c r="I91" t="str">
+        <f t="shared" si="7"/>
+        <v>pass-through</v>
+      </c>
+      <c r="J91" t="str">
+        <f t="shared" si="8"/>
+        <v>pt_methods</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>195</v>
+      </c>
+      <c r="B92" t="s">
+        <v>196</v>
+      </c>
+      <c r="C92" t="s">
+        <v>439</v>
+      </c>
+      <c r="D92" t="s">
+        <v>30</v>
+      </c>
+      <c r="E92" t="s">
+        <v>27</v>
+      </c>
+      <c r="F92" t="b">
         <v>1</v>
       </c>
-      <c r="G91" t="s">
+      <c r="G92" t="s">
         <v>21</v>
       </c>
-      <c r="H91" t="s">
+      <c r="H92" t="s">
         <v>197</v>
       </c>
-      <c r="I91" t="str">
-        <f t="shared" si="5"/>
+      <c r="I92" t="str">
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
-      <c r="J91" t="str">
-        <f t="shared" si="6"/>
+      <c r="J92" t="str">
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J91">
-    <sortCondition ref="B2:B91"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J92">
+    <sortCondition ref="B2:B92"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Remove Air Flotation ZO (#1782)
* add reference; add costing tests

* set costing year to 2007

* add validity range

* update costing test

* remove comment

* wipe air_flotation_zo from the face of the earth

* update xlsx
</commit_message>
<xml_diff>
--- a/docs/technical_reference/unit_models/zero_order_unit_models/WT3_unit_classification_for_doc.xlsx
+++ b/docs/technical_reference/unit_models/zero_order_unit_models/WT3_unit_classification_for_doc.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10531"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7C1B3F5-E496-E348-B5C9-5A5374BB4600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F101314-FCC5-314E-ADA5-DE8EBF68B42A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10580" yWindow="2740" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1200" yWindow="760" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$91</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="993" uniqueCount="511">
   <si>
     <t>Name</t>
   </si>
@@ -73,9 +73,6 @@
     <t>constant_intensity</t>
   </si>
   <si>
-    <t>air flotation</t>
-  </si>
-  <si>
     <t>air_flotation_zo</t>
   </si>
   <si>
@@ -421,6 +418,9 @@
     <t>microfiltration_zo</t>
   </si>
   <si>
+    <t>microscreen filtration</t>
+  </si>
+  <si>
     <t>microscreen_filtration_zo</t>
   </si>
   <si>
@@ -1565,18 +1565,6 @@
   </si>
   <si>
     <t>cost_electrocoagulation</t>
-  </si>
-  <si>
-    <t>crystallizer_zo</t>
-  </si>
-  <si>
-    <t>CrystallizerZO</t>
-  </si>
-  <si>
-    <t>cost_crystallizer</t>
-  </si>
-  <si>
-    <t>crystallizer</t>
   </si>
 </sst>
 </file>
@@ -1950,7 +1938,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J92"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33.5" customWidth="1"/>
@@ -2019,27 +2007,27 @@
         <v>12</v>
       </c>
       <c r="H2" t="str">
-        <f t="shared" ref="H2:H11" si="0">IF(D2="basic","cost_power_law_flow")</f>
+        <f t="shared" ref="H2:H10" si="0">IF(D2="basic","cost_power_law_flow")</f>
         <v>cost_power_law_flow</v>
       </c>
       <c r="I2" t="str">
-        <f t="shared" ref="I2:I39" si="1">IF(E2="SIDO","single-input, double-output",IF(E2="SISO","single-input, single-output",IF(E2="PT","pass-through",IF(E2="DISO","double-input, single-output",IF(E2="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
+        <f t="shared" ref="I2:I37" si="1">IF(E2="SIDO","single-input, double-output",IF(E2="SISO","single-input, single-output",IF(E2="PT","pass-through",IF(E2="DISO","double-input, single-output",IF(E2="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
         <v>single-input, double-output</v>
       </c>
       <c r="J2" t="str">
-        <f t="shared" ref="J2:J39" si="2">IF(E2="SIDO","sido_methods",IF(E2="SISO","siso_methods",IF(E2="PT","pt_methods",IF(E2="DISO","diso_methods",IF(E2="SIDO reactive","sidor_methods","")))))</f>
+        <f t="shared" ref="J2:J37" si="2">IF(E2="SIDO","sido_methods",IF(E2="SISO","siso_methods",IF(E2="PT","pt_methods",IF(E2="DISO","diso_methods",IF(E2="SIDO reactive","sidor_methods","")))))</f>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>505</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>383</v>
+        <v>421</v>
       </c>
       <c r="D3" t="s">
         <v>10</v>
@@ -2054,7 +2042,7 @@
         <v>12</v>
       </c>
       <c r="H3" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(D3="basic","cost_power_law_flow")</f>
         <v>cost_power_law_flow</v>
       </c>
       <c r="I3" t="str">
@@ -2068,19 +2056,19 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>505</v>
+        <v>462</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>463</v>
       </c>
       <c r="C4" t="s">
-        <v>421</v>
+        <v>461</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -2088,43 +2076,42 @@
       <c r="G4" t="s">
         <v>12</v>
       </c>
-      <c r="H4" t="str">
-        <f>IF(D4="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H4" t="s">
+        <v>64</v>
       </c>
       <c r="I4" t="str">
         <f t="shared" si="1"/>
-        <v>single-input, double-output</v>
+        <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J4" t="str">
         <f t="shared" si="2"/>
-        <v>sido_methods</v>
+        <v>sidor_methods</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>462</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>463</v>
+        <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>461</v>
+        <v>445</v>
       </c>
       <c r="D5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H5" t="s">
-        <v>65</v>
+        <v>457</v>
       </c>
       <c r="I5" t="str">
         <f t="shared" si="1"/>
@@ -2137,28 +2124,28 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>464</v>
       </c>
       <c r="B6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C6" t="s">
+        <v>446</v>
+      </c>
+      <c r="D6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" t="s">
         <v>17</v>
       </c>
-      <c r="C6" t="s">
-        <v>445</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="F6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" t="s">
         <v>30</v>
       </c>
-      <c r="E6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G6" t="s">
-        <v>21</v>
-      </c>
       <c r="H6" t="s">
-        <v>457</v>
+        <v>465</v>
       </c>
       <c r="I6" t="str">
         <f t="shared" si="1"/>
@@ -2171,47 +2158,48 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>464</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>454</v>
+        <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>446</v>
+        <v>374</v>
       </c>
       <c r="D7" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>31</v>
-      </c>
-      <c r="H7" t="s">
-        <v>465</v>
+        <v>20</v>
+      </c>
+      <c r="H7" t="str">
+        <f t="shared" si="0"/>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I7" t="str">
         <f t="shared" si="1"/>
-        <v>reactive single-inlet, double-outlet</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J7" t="str">
         <f t="shared" si="2"/>
-        <v>sidor_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -2223,7 +2211,7 @@
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="H8" t="str">
         <f t="shared" si="0"/>
@@ -2240,19 +2228,19 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>375</v>
+        <v>384</v>
       </c>
       <c r="D9" t="s">
         <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
@@ -2266,22 +2254,22 @@
       </c>
       <c r="I9" t="str">
         <f t="shared" si="1"/>
-        <v>single-input, double-output</v>
+        <v>single-input, single-output</v>
       </c>
       <c r="J9" t="str">
         <f t="shared" si="2"/>
-        <v>sido_methods</v>
+        <v>siso_methods</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>371</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>370</v>
       </c>
       <c r="C10" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
@@ -2301,163 +2289,163 @@
       </c>
       <c r="I10" t="str">
         <f t="shared" si="1"/>
-        <v>single-input, single-output</v>
+        <v>pass-through</v>
       </c>
       <c r="J10" t="str">
         <f t="shared" si="2"/>
-        <v>siso_methods</v>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>371</v>
+        <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>370</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>376</v>
+        <v>427</v>
       </c>
       <c r="D11" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E11" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="s">
-        <v>12</v>
-      </c>
-      <c r="H11" t="str">
-        <f t="shared" si="0"/>
-        <v>cost_power_law_flow</v>
+        <v>30</v>
+      </c>
+      <c r="H11" t="s">
+        <v>31</v>
       </c>
       <c r="I11" t="str">
         <f t="shared" si="1"/>
-        <v>pass-through</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J11" t="str">
         <f t="shared" si="2"/>
-        <v>pt_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C12" t="s">
-        <v>427</v>
+        <v>386</v>
       </c>
       <c r="D12" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E12" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="s">
-        <v>31</v>
-      </c>
-      <c r="H12" t="s">
-        <v>32</v>
+        <v>12</v>
+      </c>
+      <c r="H12" t="str">
+        <f>IF(D12="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I12" t="str">
         <f t="shared" si="1"/>
-        <v>single-input, double-output</v>
+        <v>pass-through</v>
       </c>
       <c r="J12" t="str">
         <f t="shared" si="2"/>
-        <v>sido_methods</v>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>386</v>
+        <v>444</v>
       </c>
       <c r="D13" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E13" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" t="s">
-        <v>12</v>
-      </c>
-      <c r="H13" t="str">
-        <f>IF(D13="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>30</v>
+      </c>
+      <c r="H13" t="s">
+        <v>36</v>
       </c>
       <c r="I13" t="str">
         <f t="shared" si="1"/>
-        <v>pass-through</v>
+        <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J13" t="str">
         <f t="shared" si="2"/>
-        <v>pt_methods</v>
+        <v>sidor_methods</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C14" t="s">
-        <v>444</v>
+        <v>388</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E14" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" t="s">
-        <v>31</v>
-      </c>
-      <c r="H14" t="s">
-        <v>37</v>
+        <v>12</v>
+      </c>
+      <c r="H14" t="str">
+        <f>IF(D14="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I14" t="str">
         <f t="shared" si="1"/>
-        <v>reactive single-inlet, double-outlet</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J14" t="str">
         <f t="shared" si="2"/>
-        <v>sidor_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>466</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
+        <v>467</v>
       </c>
       <c r="C15" t="s">
-        <v>388</v>
+        <v>468</v>
       </c>
       <c r="D15" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E15" t="s">
         <v>11</v>
@@ -2468,9 +2456,8 @@
       <c r="G15" t="s">
         <v>12</v>
       </c>
-      <c r="H15" t="str">
-        <f>IF(D15="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H15" t="s">
+        <v>469</v>
       </c>
       <c r="I15" t="str">
         <f t="shared" si="1"/>
@@ -2483,87 +2470,87 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>466</v>
+        <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>467</v>
+        <v>40</v>
       </c>
       <c r="C16" t="s">
-        <v>468</v>
+        <v>387</v>
       </c>
       <c r="D16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" t="b">
+        <v>0</v>
+      </c>
+      <c r="G16" t="s">
         <v>30</v>
       </c>
-      <c r="E16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F16" t="b">
-        <v>1</v>
-      </c>
-      <c r="G16" t="s">
-        <v>12</v>
-      </c>
       <c r="H16" t="s">
-        <v>469</v>
+        <v>41</v>
       </c>
       <c r="I16" t="str">
         <f t="shared" si="1"/>
-        <v>single-input, double-output</v>
+        <v>pass-through</v>
       </c>
       <c r="J16" t="str">
         <f t="shared" si="2"/>
-        <v>sido_methods</v>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>387</v>
+        <v>432</v>
       </c>
       <c r="D17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E17" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H17" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I17" t="str">
         <f t="shared" si="1"/>
-        <v>pass-through</v>
+        <v>single-input, single-output</v>
       </c>
       <c r="J17" t="str">
         <f t="shared" si="2"/>
-        <v>pt_methods</v>
+        <v>siso_methods</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>432</v>
+        <v>406</v>
       </c>
       <c r="D18" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E18" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F18" t="b">
         <v>1</v>
@@ -2571,27 +2558,28 @@
       <c r="G18" t="s">
         <v>12</v>
       </c>
-      <c r="H18" t="s">
-        <v>45</v>
+      <c r="H18" t="str">
+        <f>IF(D18="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I18" t="str">
         <f t="shared" si="1"/>
-        <v>single-input, single-output</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J18" t="str">
         <f t="shared" si="2"/>
-        <v>siso_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>46</v>
+        <v>470</v>
       </c>
       <c r="B19" t="s">
-        <v>47</v>
+        <v>471</v>
       </c>
       <c r="C19" t="s">
-        <v>406</v>
+        <v>472</v>
       </c>
       <c r="D19" t="s">
         <v>10</v>
@@ -2605,9 +2593,8 @@
       <c r="G19" t="s">
         <v>12</v>
       </c>
-      <c r="H19" t="str">
-        <f>IF(D19="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H19" t="s">
+        <v>64</v>
       </c>
       <c r="I19" t="str">
         <f t="shared" si="1"/>
@@ -2620,19 +2607,19 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>470</v>
+        <v>47</v>
       </c>
       <c r="B20" t="s">
-        <v>471</v>
+        <v>48</v>
       </c>
       <c r="C20" t="s">
-        <v>472</v>
+        <v>434</v>
       </c>
       <c r="D20" t="s">
         <v>10</v>
       </c>
       <c r="E20" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F20" t="b">
         <v>1</v>
@@ -2640,43 +2627,43 @@
       <c r="G20" t="s">
         <v>12</v>
       </c>
-      <c r="H20" t="s">
-        <v>65</v>
+      <c r="H20" t="str">
+        <f>IF(D20="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I20" t="str">
         <f t="shared" si="1"/>
-        <v>single-input, double-output</v>
+        <v>pass-through</v>
       </c>
       <c r="J20" t="str">
         <f t="shared" si="2"/>
-        <v>sido_methods</v>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C21" t="s">
-        <v>434</v>
+        <v>415</v>
       </c>
       <c r="D21" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" t="s">
-        <v>12</v>
-      </c>
-      <c r="H21" t="str">
-        <f>IF(D21="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>30</v>
+      </c>
+      <c r="H21" t="s">
+        <v>51</v>
       </c>
       <c r="I21" t="str">
         <f t="shared" si="1"/>
@@ -2689,121 +2676,122 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B22" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C22" t="s">
-        <v>415</v>
+        <v>448</v>
       </c>
       <c r="D22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E22" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H22" t="s">
-        <v>52</v>
+        <v>458</v>
       </c>
       <c r="I22" t="str">
         <f t="shared" si="1"/>
-        <v>pass-through</v>
+        <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J22" t="str">
         <f t="shared" si="2"/>
-        <v>pt_methods</v>
+        <v>sidor_methods</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B23" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C23" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E23" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" t="s">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="H23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="I23" t="str">
         <f t="shared" si="1"/>
-        <v>reactive single-inlet, double-outlet</v>
+        <v>single-input, single-output</v>
       </c>
       <c r="J23" t="str">
         <f t="shared" si="2"/>
-        <v>sidor_methods</v>
+        <v>siso_methods</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C24" t="s">
-        <v>449</v>
+        <v>377</v>
       </c>
       <c r="D24" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E24" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" t="s">
-        <v>58</v>
-      </c>
-      <c r="H24" t="s">
-        <v>459</v>
+        <v>12</v>
+      </c>
+      <c r="H24" t="str">
+        <f>IF(D24="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I24" t="str">
         <f t="shared" si="1"/>
-        <v>single-input, single-output</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J24" t="str">
         <f t="shared" si="2"/>
-        <v>siso_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B25" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C25" t="s">
-        <v>377</v>
+        <v>389</v>
       </c>
       <c r="D25" t="s">
         <v>10</v>
       </c>
       <c r="E25" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F25" t="b">
         <v>1</v>
@@ -2817,28 +2805,28 @@
       </c>
       <c r="I25" t="str">
         <f t="shared" si="1"/>
-        <v>single-input, double-output</v>
+        <v>pass-through</v>
       </c>
       <c r="J25" t="str">
         <f t="shared" si="2"/>
-        <v>sido_methods</v>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B26" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C26" t="s">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="D26" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E26" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F26" t="b">
         <v>1</v>
@@ -2846,34 +2834,33 @@
       <c r="G26" t="s">
         <v>12</v>
       </c>
-      <c r="H26" t="str">
-        <f>IF(D26="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H26" t="s">
+        <v>64</v>
       </c>
       <c r="I26" t="str">
         <f t="shared" si="1"/>
-        <v>pass-through</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J26" t="str">
         <f t="shared" si="2"/>
-        <v>pt_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B27" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C27" t="s">
-        <v>378</v>
+        <v>390</v>
       </c>
       <c r="D27" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E27" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F27" t="b">
         <v>1</v>
@@ -2881,67 +2868,68 @@
       <c r="G27" t="s">
         <v>12</v>
       </c>
-      <c r="H27" t="s">
-        <v>65</v>
+      <c r="H27" t="str">
+        <f>IF(D27="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I27" t="str">
         <f t="shared" si="1"/>
-        <v>single-input, double-output</v>
+        <v>single-input, single-output</v>
       </c>
       <c r="J27" t="str">
         <f t="shared" si="2"/>
-        <v>sido_methods</v>
+        <v>siso_methods</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>514</v>
+        <v>67</v>
       </c>
       <c r="B28" t="s">
-        <v>511</v>
+        <v>68</v>
       </c>
       <c r="C28" t="s">
-        <v>512</v>
+        <v>379</v>
       </c>
       <c r="D28" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E28" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G28" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H28" t="s">
-        <v>513</v>
+        <v>69</v>
       </c>
       <c r="I28" t="str">
-        <f t="shared" ref="I28" si="3">IF(E28="SIDO","single-input, double-output",IF(E28="SISO","single-input, single-output",IF(E28="PT","pass-through",IF(E28="DISO","double-input, single-output",IF(E28="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
-        <v>single-input, double-output</v>
+        <f t="shared" si="1"/>
+        <v>pass-through</v>
       </c>
       <c r="J28" t="str">
-        <f t="shared" ref="J28" si="4">IF(E28="SIDO","sido_methods",IF(E28="SISO","siso_methods",IF(E28="PT","pt_methods",IF(E28="DISO","diso_methods",IF(E28="SIDO reactive","sidor_methods","")))))</f>
-        <v>sido_methods</v>
+        <f t="shared" si="2"/>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B29" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C29" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D29" t="s">
         <v>10</v>
       </c>
       <c r="E29" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F29" t="b">
         <v>1</v>
@@ -2955,56 +2943,56 @@
       </c>
       <c r="I29" t="str">
         <f t="shared" si="1"/>
-        <v>single-input, single-output</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J29" t="str">
         <f t="shared" si="2"/>
-        <v>siso_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B30" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C30" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D30" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="E30" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F30" t="b">
         <v>1</v>
       </c>
       <c r="G30" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="H30" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="I30" t="str">
         <f t="shared" si="1"/>
-        <v>pass-through</v>
+        <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J30" t="str">
         <f t="shared" si="2"/>
-        <v>pt_methods</v>
+        <v>sidor_methods</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B31" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C31" t="s">
-        <v>391</v>
+        <v>429</v>
       </c>
       <c r="D31" t="s">
         <v>10</v>
@@ -3033,28 +3021,28 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B32" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C32" t="s">
-        <v>380</v>
+        <v>394</v>
       </c>
       <c r="D32" t="s">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="E32" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="H32" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="I32" t="str">
         <f t="shared" si="1"/>
@@ -3067,29 +3055,28 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>76</v>
+        <v>507</v>
       </c>
       <c r="B33" t="s">
-        <v>77</v>
+        <v>508</v>
       </c>
       <c r="C33" t="s">
-        <v>429</v>
+        <v>509</v>
       </c>
       <c r="D33" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E33" t="s">
         <v>11</v>
       </c>
       <c r="F33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33" t="s">
-        <v>12</v>
-      </c>
-      <c r="H33" t="str">
-        <f>IF(D33="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>30</v>
+      </c>
+      <c r="H33" t="s">
+        <v>510</v>
       </c>
       <c r="I33" t="str">
         <f t="shared" si="1"/>
@@ -3102,96 +3089,97 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B34" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C34" t="s">
-        <v>394</v>
+        <v>381</v>
       </c>
       <c r="D34" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E34" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F34" t="b">
         <v>0</v>
       </c>
       <c r="G34" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H34" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="I34" t="str">
         <f t="shared" si="1"/>
-        <v>reactive single-inlet, double-outlet</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J34" t="str">
         <f t="shared" si="2"/>
-        <v>sidor_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>507</v>
+        <v>82</v>
       </c>
       <c r="B35" t="s">
-        <v>508</v>
+        <v>83</v>
       </c>
       <c r="C35" t="s">
-        <v>509</v>
+        <v>395</v>
       </c>
       <c r="D35" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E35" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G35" t="s">
-        <v>31</v>
-      </c>
-      <c r="H35" t="s">
-        <v>510</v>
+        <v>12</v>
+      </c>
+      <c r="H35" t="str">
+        <f>IF(D35="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I35" t="str">
         <f t="shared" si="1"/>
-        <v>single-input, double-output</v>
+        <v>pass-through</v>
       </c>
       <c r="J35" t="str">
         <f t="shared" si="2"/>
-        <v>sido_methods</v>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B36" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C36" t="s">
-        <v>381</v>
+        <v>436</v>
       </c>
       <c r="D36" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E36" t="s">
         <v>11</v>
       </c>
       <c r="F36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H36" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="I36" t="str">
         <f t="shared" si="1"/>
@@ -3204,19 +3192,19 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B37" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C37" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="D37" t="s">
         <v>10</v>
       </c>
       <c r="E37" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F37" t="b">
         <v>1</v>
@@ -3239,118 +3227,117 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B38" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C38" t="s">
-        <v>436</v>
+        <v>393</v>
       </c>
       <c r="D38" t="s">
-        <v>30</v>
+        <v>91</v>
       </c>
       <c r="E38" t="s">
-        <v>11</v>
+        <v>57</v>
       </c>
       <c r="F38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G38" t="s">
-        <v>12</v>
-      </c>
-      <c r="H38" t="s">
-        <v>87</v>
-      </c>
-      <c r="I38" t="str">
-        <f t="shared" si="1"/>
-        <v>single-input, double-output</v>
-      </c>
-      <c r="J38" t="str">
-        <f t="shared" si="2"/>
-        <v>sido_methods</v>
+        <v>57</v>
+      </c>
+      <c r="H38" t="b">
+        <f>IF(D38="basic","cost_power_law_flow")</f>
+        <v>0</v>
+      </c>
+      <c r="I38" t="s">
+        <v>92</v>
+      </c>
+      <c r="J38" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B39" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C39" t="s">
-        <v>392</v>
+        <v>437</v>
       </c>
       <c r="D39" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E39" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G39" t="s">
-        <v>12</v>
-      </c>
-      <c r="H39" t="str">
-        <f>IF(D39="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>30</v>
+      </c>
+      <c r="H39" t="s">
+        <v>95</v>
       </c>
       <c r="I39" t="str">
-        <f t="shared" si="1"/>
-        <v>pass-through</v>
+        <f t="shared" ref="I39:I44" si="3">IF(E39="SIDO","single-input, double-output",IF(E39="SISO","single-input, single-output",IF(E39="PT","pass-through",IF(E39="DISO","double-input, single-output",IF(E39="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
+        <v>single-input, double-output</v>
       </c>
       <c r="J39" t="str">
-        <f t="shared" si="2"/>
-        <v>pt_methods</v>
+        <f t="shared" ref="J39:J44" si="4">IF(E39="SIDO","sido_methods",IF(E39="SISO","siso_methods",IF(E39="PT","pt_methods",IF(E39="DISO","diso_methods",IF(E39="SIDO reactive","sidor_methods","")))))</f>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B40" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C40" t="s">
-        <v>393</v>
+        <v>422</v>
       </c>
       <c r="D40" t="s">
-        <v>92</v>
+        <v>29</v>
       </c>
       <c r="E40" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="F40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" t="s">
-        <v>58</v>
-      </c>
-      <c r="H40" t="b">
-        <f>IF(D40="basic","cost_power_law_flow")</f>
-        <v>0</v>
-      </c>
-      <c r="I40" t="s">
-        <v>93</v>
-      </c>
-      <c r="J40" t="s">
-        <v>93</v>
+        <v>12</v>
+      </c>
+      <c r="H40" t="s">
+        <v>98</v>
+      </c>
+      <c r="I40" t="str">
+        <f t="shared" si="3"/>
+        <v>single-input, single-output</v>
+      </c>
+      <c r="J40" t="str">
+        <f t="shared" si="4"/>
+        <v>siso_methods</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B41" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C41" t="s">
-        <v>437</v>
+        <v>428</v>
       </c>
       <c r="D41" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E41" t="s">
         <v>11</v>
@@ -3359,960 +3346,962 @@
         <v>0</v>
       </c>
       <c r="G41" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H41" t="s">
-        <v>96</v>
+        <v>506</v>
       </c>
       <c r="I41" t="str">
-        <f t="shared" ref="I41:I46" si="5">IF(E41="SIDO","single-input, double-output",IF(E41="SISO","single-input, single-output",IF(E41="PT","pass-through",IF(E41="DISO","double-input, single-output",IF(E41="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
+        <f t="shared" si="3"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J41" t="str">
-        <f t="shared" ref="J41:J46" si="6">IF(E41="SIDO","sido_methods",IF(E41="SISO","siso_methods",IF(E41="PT","pt_methods",IF(E41="DISO","diso_methods",IF(E41="SIDO reactive","sidor_methods","")))))</f>
+        <f t="shared" si="4"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B42" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C42" t="s">
-        <v>422</v>
+        <v>450</v>
       </c>
       <c r="D42" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E42" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F42" t="b">
         <v>1</v>
       </c>
       <c r="G42" t="s">
+        <v>20</v>
+      </c>
+      <c r="H42" t="b">
+        <v>0</v>
+      </c>
+      <c r="I42" t="str">
+        <f t="shared" si="3"/>
+        <v>single-input, double-output</v>
+      </c>
+      <c r="J42" t="str">
+        <f t="shared" si="4"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>474</v>
+      </c>
+      <c r="B43" t="s">
+        <v>473</v>
+      </c>
+      <c r="C43" t="s">
+        <v>475</v>
+      </c>
+      <c r="D43" t="s">
+        <v>10</v>
+      </c>
+      <c r="E43" t="s">
+        <v>17</v>
+      </c>
+      <c r="F43" t="b">
+        <v>1</v>
+      </c>
+      <c r="G43" t="s">
         <v>12</v>
       </c>
-      <c r="H42" t="s">
-        <v>99</v>
-      </c>
-      <c r="I42" t="str">
+      <c r="H43" t="s">
+        <v>476</v>
+      </c>
+      <c r="I43" t="str">
+        <f t="shared" si="3"/>
+        <v>reactive single-inlet, double-outlet</v>
+      </c>
+      <c r="J43" t="str">
+        <f t="shared" si="4"/>
+        <v>sidor_methods</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>477</v>
+      </c>
+      <c r="B44" t="s">
+        <v>455</v>
+      </c>
+      <c r="C44" t="s">
+        <v>451</v>
+      </c>
+      <c r="D44" t="s">
+        <v>29</v>
+      </c>
+      <c r="E44" t="s">
+        <v>17</v>
+      </c>
+      <c r="F44" t="b">
+        <v>1</v>
+      </c>
+      <c r="G44" t="s">
+        <v>30</v>
+      </c>
+      <c r="H44" t="s">
+        <v>478</v>
+      </c>
+      <c r="I44" t="str">
+        <f t="shared" si="3"/>
+        <v>reactive single-inlet, double-outlet</v>
+      </c>
+      <c r="J44" t="str">
+        <f t="shared" si="4"/>
+        <v>sidor_methods</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>103</v>
+      </c>
+      <c r="B45" t="s">
+        <v>104</v>
+      </c>
+      <c r="C45" t="s">
+        <v>441</v>
+      </c>
+      <c r="D45" t="s">
+        <v>10</v>
+      </c>
+      <c r="E45" t="s">
+        <v>26</v>
+      </c>
+      <c r="F45" t="b">
+        <v>1</v>
+      </c>
+      <c r="G45" t="s">
+        <v>12</v>
+      </c>
+      <c r="H45" t="str">
+        <f>IF(D45="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
+      </c>
+      <c r="I45" t="str">
+        <f t="shared" ref="I45:I91" si="5">IF(E45="SIDO","single-input, double-output",IF(E45="SISO","single-input, single-output",IF(E45="PT","pass-through",IF(E45="DISO","double-input, single-output",IF(E45="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
+        <v>pass-through</v>
+      </c>
+      <c r="J45" t="str">
+        <f t="shared" ref="J45:J91" si="6">IF(E45="SIDO","sido_methods",IF(E45="SISO","siso_methods",IF(E45="PT","pt_methods",IF(E45="DISO","diso_methods",IF(E45="SIDO reactive","sidor_methods","")))))</f>
+        <v>pt_methods</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>105</v>
+      </c>
+      <c r="B46" t="s">
+        <v>106</v>
+      </c>
+      <c r="C46" t="s">
+        <v>440</v>
+      </c>
+      <c r="D46" t="s">
+        <v>10</v>
+      </c>
+      <c r="E46" t="s">
+        <v>26</v>
+      </c>
+      <c r="F46" t="b">
+        <v>1</v>
+      </c>
+      <c r="G46" t="s">
+        <v>12</v>
+      </c>
+      <c r="H46" t="str">
+        <f>IF(D46="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
+      </c>
+      <c r="I46" t="str">
+        <f t="shared" si="5"/>
+        <v>pass-through</v>
+      </c>
+      <c r="J46" t="str">
+        <f t="shared" si="6"/>
+        <v>pt_methods</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>107</v>
+      </c>
+      <c r="B47" t="s">
+        <v>108</v>
+      </c>
+      <c r="C47" t="s">
+        <v>426</v>
+      </c>
+      <c r="D47" t="s">
+        <v>29</v>
+      </c>
+      <c r="E47" t="s">
+        <v>11</v>
+      </c>
+      <c r="F47" t="b">
+        <v>1</v>
+      </c>
+      <c r="G47" t="s">
+        <v>20</v>
+      </c>
+      <c r="H47" t="s">
+        <v>109</v>
+      </c>
+      <c r="I47" t="str">
+        <f t="shared" si="5"/>
+        <v>single-input, double-output</v>
+      </c>
+      <c r="J47" t="str">
+        <f t="shared" si="6"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>110</v>
+      </c>
+      <c r="B48" t="s">
+        <v>111</v>
+      </c>
+      <c r="C48" t="s">
+        <v>396</v>
+      </c>
+      <c r="D48" t="s">
+        <v>29</v>
+      </c>
+      <c r="E48" t="s">
+        <v>11</v>
+      </c>
+      <c r="F48" t="b">
+        <v>0</v>
+      </c>
+      <c r="G48" t="s">
+        <v>30</v>
+      </c>
+      <c r="H48" t="s">
+        <v>112</v>
+      </c>
+      <c r="I48" t="str">
+        <f t="shared" si="5"/>
+        <v>single-input, double-output</v>
+      </c>
+      <c r="J48" t="str">
+        <f t="shared" si="6"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>113</v>
+      </c>
+      <c r="B49" t="s">
+        <v>114</v>
+      </c>
+      <c r="C49" t="s">
+        <v>397</v>
+      </c>
+      <c r="D49" t="s">
+        <v>10</v>
+      </c>
+      <c r="E49" t="s">
+        <v>26</v>
+      </c>
+      <c r="F49" t="b">
+        <v>1</v>
+      </c>
+      <c r="G49" t="s">
+        <v>12</v>
+      </c>
+      <c r="H49" t="s">
+        <v>115</v>
+      </c>
+      <c r="I49" t="str">
+        <f t="shared" si="5"/>
+        <v>pass-through</v>
+      </c>
+      <c r="J49" t="str">
+        <f t="shared" si="6"/>
+        <v>pt_methods</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>116</v>
+      </c>
+      <c r="B50" t="s">
+        <v>117</v>
+      </c>
+      <c r="C50" t="s">
+        <v>399</v>
+      </c>
+      <c r="D50" t="s">
+        <v>29</v>
+      </c>
+      <c r="E50" t="s">
+        <v>17</v>
+      </c>
+      <c r="F50" t="b">
+        <v>1</v>
+      </c>
+      <c r="G50" t="s">
+        <v>12</v>
+      </c>
+      <c r="H50" t="s">
+        <v>118</v>
+      </c>
+      <c r="I50" t="str">
+        <f t="shared" si="5"/>
+        <v>reactive single-inlet, double-outlet</v>
+      </c>
+      <c r="J50" t="str">
+        <f t="shared" si="6"/>
+        <v>sidor_methods</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>479</v>
+      </c>
+      <c r="B51" t="s">
+        <v>480</v>
+      </c>
+      <c r="C51" t="s">
+        <v>481</v>
+      </c>
+      <c r="D51" t="s">
+        <v>29</v>
+      </c>
+      <c r="E51" t="s">
+        <v>17</v>
+      </c>
+      <c r="F51" t="b">
+        <v>1</v>
+      </c>
+      <c r="G51" t="s">
+        <v>12</v>
+      </c>
+      <c r="H51" t="s">
+        <v>482</v>
+      </c>
+      <c r="I51" t="str">
+        <f t="shared" si="5"/>
+        <v>reactive single-inlet, double-outlet</v>
+      </c>
+      <c r="J51" t="str">
+        <f t="shared" si="6"/>
+        <v>sidor_methods</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>119</v>
+      </c>
+      <c r="B52" t="s">
+        <v>120</v>
+      </c>
+      <c r="C52" t="s">
+        <v>400</v>
+      </c>
+      <c r="D52" t="s">
+        <v>10</v>
+      </c>
+      <c r="E52" t="s">
+        <v>11</v>
+      </c>
+      <c r="F52" t="b">
+        <v>1</v>
+      </c>
+      <c r="G52" t="s">
+        <v>12</v>
+      </c>
+      <c r="H52" t="str">
+        <f>IF(D52="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
+      </c>
+      <c r="I52" t="str">
+        <f t="shared" si="5"/>
+        <v>single-input, double-output</v>
+      </c>
+      <c r="J52" t="str">
+        <f t="shared" si="6"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>121</v>
+      </c>
+      <c r="B53" t="s">
+        <v>122</v>
+      </c>
+      <c r="C53" t="s">
+        <v>401</v>
+      </c>
+      <c r="D53" t="s">
+        <v>10</v>
+      </c>
+      <c r="E53" t="s">
+        <v>11</v>
+      </c>
+      <c r="F53" t="b">
+        <v>1</v>
+      </c>
+      <c r="G53" t="s">
+        <v>12</v>
+      </c>
+      <c r="H53" t="str">
+        <f>IF(D53="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
+      </c>
+      <c r="I53" t="str">
+        <f t="shared" si="5"/>
+        <v>single-input, double-output</v>
+      </c>
+      <c r="J53" t="str">
+        <f t="shared" si="6"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>483</v>
+      </c>
+      <c r="B54" t="s">
+        <v>484</v>
+      </c>
+      <c r="C54" t="s">
+        <v>485</v>
+      </c>
+      <c r="D54" t="s">
+        <v>29</v>
+      </c>
+      <c r="E54" t="s">
+        <v>11</v>
+      </c>
+      <c r="F54" t="b">
+        <v>1</v>
+      </c>
+      <c r="G54" t="s">
+        <v>12</v>
+      </c>
+      <c r="H54" t="s">
+        <v>486</v>
+      </c>
+      <c r="I54" t="str">
+        <f t="shared" si="5"/>
+        <v>single-input, double-output</v>
+      </c>
+      <c r="J54" t="str">
+        <f t="shared" si="6"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>123</v>
+      </c>
+      <c r="B55" t="s">
+        <v>124</v>
+      </c>
+      <c r="C55" t="s">
+        <v>385</v>
+      </c>
+      <c r="D55" t="s">
+        <v>29</v>
+      </c>
+      <c r="E55" t="s">
+        <v>17</v>
+      </c>
+      <c r="F55" t="b">
+        <v>0</v>
+      </c>
+      <c r="G55" t="s">
+        <v>30</v>
+      </c>
+      <c r="H55" t="s">
+        <v>125</v>
+      </c>
+      <c r="I55" t="str">
+        <f t="shared" si="5"/>
+        <v>reactive single-inlet, double-outlet</v>
+      </c>
+      <c r="J55" t="str">
+        <f t="shared" si="6"/>
+        <v>sidor_methods</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>487</v>
+      </c>
+      <c r="B56" t="s">
+        <v>488</v>
+      </c>
+      <c r="C56" t="s">
+        <v>489</v>
+      </c>
+      <c r="D56" t="s">
+        <v>29</v>
+      </c>
+      <c r="E56" t="s">
+        <v>17</v>
+      </c>
+      <c r="F56" t="b">
+        <v>1</v>
+      </c>
+      <c r="G56" t="s">
+        <v>12</v>
+      </c>
+      <c r="H56" t="s">
+        <v>490</v>
+      </c>
+      <c r="I56" t="str">
+        <f t="shared" si="5"/>
+        <v>reactive single-inlet, double-outlet</v>
+      </c>
+      <c r="J56" t="str">
+        <f t="shared" si="6"/>
+        <v>sidor_methods</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>126</v>
+      </c>
+      <c r="B57" t="s">
+        <v>127</v>
+      </c>
+      <c r="C57" t="s">
+        <v>402</v>
+      </c>
+      <c r="D57" t="s">
+        <v>10</v>
+      </c>
+      <c r="E57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F57" t="b">
+        <v>1</v>
+      </c>
+      <c r="G57" t="s">
+        <v>12</v>
+      </c>
+      <c r="H57" t="str">
+        <f>IF(D57="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
+      </c>
+      <c r="I57" t="str">
+        <f t="shared" si="5"/>
+        <v>single-input, double-output</v>
+      </c>
+      <c r="J57" t="str">
+        <f t="shared" si="6"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>128</v>
+      </c>
+      <c r="B58" t="s">
+        <v>129</v>
+      </c>
+      <c r="C58" t="s">
+        <v>403</v>
+      </c>
+      <c r="D58" t="s">
+        <v>10</v>
+      </c>
+      <c r="E58" t="s">
+        <v>11</v>
+      </c>
+      <c r="F58" t="b">
+        <v>1</v>
+      </c>
+      <c r="G58" t="s">
+        <v>12</v>
+      </c>
+      <c r="H58" t="str">
+        <f>IF(D58="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
+      </c>
+      <c r="I58" t="str">
+        <f t="shared" si="5"/>
+        <v>single-input, double-output</v>
+      </c>
+      <c r="J58" t="str">
+        <f t="shared" si="6"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>130</v>
+      </c>
+      <c r="B59" t="s">
+        <v>131</v>
+      </c>
+      <c r="C59" t="s">
+        <v>423</v>
+      </c>
+      <c r="D59" t="s">
+        <v>10</v>
+      </c>
+      <c r="E59" t="s">
+        <v>26</v>
+      </c>
+      <c r="F59" t="b">
+        <v>1</v>
+      </c>
+      <c r="G59" t="s">
+        <v>20</v>
+      </c>
+      <c r="H59" t="s">
+        <v>64</v>
+      </c>
+      <c r="I59" t="str">
+        <f t="shared" si="5"/>
+        <v>pass-through</v>
+      </c>
+      <c r="J59" t="str">
+        <f t="shared" si="6"/>
+        <v>pt_methods</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>132</v>
+      </c>
+      <c r="B60" t="s">
+        <v>133</v>
+      </c>
+      <c r="C60" t="s">
+        <v>404</v>
+      </c>
+      <c r="D60" t="s">
+        <v>10</v>
+      </c>
+      <c r="E60" t="s">
+        <v>26</v>
+      </c>
+      <c r="F60" t="b">
+        <v>1</v>
+      </c>
+      <c r="G60" t="s">
+        <v>12</v>
+      </c>
+      <c r="H60" t="str">
+        <f>IF(D60="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
+      </c>
+      <c r="I60" t="str">
+        <f t="shared" si="5"/>
+        <v>pass-through</v>
+      </c>
+      <c r="J60" t="str">
+        <f t="shared" si="6"/>
+        <v>pt_methods</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>134</v>
+      </c>
+      <c r="B61" t="s">
+        <v>135</v>
+      </c>
+      <c r="C61" t="s">
+        <v>405</v>
+      </c>
+      <c r="D61" t="s">
+        <v>29</v>
+      </c>
+      <c r="E61" t="s">
+        <v>11</v>
+      </c>
+      <c r="F61" t="b">
+        <v>0</v>
+      </c>
+      <c r="G61" t="s">
+        <v>30</v>
+      </c>
+      <c r="H61" t="s">
+        <v>136</v>
+      </c>
+      <c r="I61" t="str">
+        <f t="shared" si="5"/>
+        <v>single-input, double-output</v>
+      </c>
+      <c r="J61" t="str">
+        <f t="shared" si="6"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>137</v>
+      </c>
+      <c r="B62" t="s">
+        <v>369</v>
+      </c>
+      <c r="C62" t="s">
+        <v>425</v>
+      </c>
+      <c r="D62" t="s">
+        <v>29</v>
+      </c>
+      <c r="E62" t="s">
+        <v>25</v>
+      </c>
+      <c r="F62" t="b">
+        <v>0</v>
+      </c>
+      <c r="G62" t="s">
+        <v>30</v>
+      </c>
+      <c r="H62" t="s">
+        <v>138</v>
+      </c>
+      <c r="I62" t="str">
         <f t="shared" si="5"/>
         <v>single-input, single-output</v>
       </c>
-      <c r="J42" t="str">
+      <c r="J62" t="str">
         <f t="shared" si="6"/>
         <v>siso_methods</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>100</v>
-      </c>
-      <c r="B43" t="s">
-        <v>101</v>
-      </c>
-      <c r="C43" t="s">
-        <v>428</v>
-      </c>
-      <c r="D43" t="s">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>139</v>
+      </c>
+      <c r="B63" t="s">
+        <v>140</v>
+      </c>
+      <c r="C63" t="s">
+        <v>424</v>
+      </c>
+      <c r="D63" t="s">
+        <v>29</v>
+      </c>
+      <c r="E63" t="s">
+        <v>25</v>
+      </c>
+      <c r="F63" t="b">
+        <v>0</v>
+      </c>
+      <c r="G63" t="s">
         <v>30</v>
       </c>
-      <c r="E43" t="s">
+      <c r="H63" t="s">
+        <v>141</v>
+      </c>
+      <c r="I63" t="str">
+        <f t="shared" si="5"/>
+        <v>single-input, single-output</v>
+      </c>
+      <c r="J63" t="str">
+        <f t="shared" si="6"/>
+        <v>siso_methods</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>491</v>
+      </c>
+      <c r="B64" t="s">
+        <v>492</v>
+      </c>
+      <c r="C64" t="s">
+        <v>493</v>
+      </c>
+      <c r="D64" t="s">
+        <v>29</v>
+      </c>
+      <c r="E64" t="s">
+        <v>17</v>
+      </c>
+      <c r="F64" t="b">
+        <v>1</v>
+      </c>
+      <c r="G64" t="s">
+        <v>12</v>
+      </c>
+      <c r="H64" t="s">
+        <v>494</v>
+      </c>
+      <c r="I64" t="str">
+        <f t="shared" si="5"/>
+        <v>reactive single-inlet, double-outlet</v>
+      </c>
+      <c r="J64" t="str">
+        <f t="shared" si="6"/>
+        <v>sidor_methods</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>142</v>
+      </c>
+      <c r="B65" t="s">
+        <v>143</v>
+      </c>
+      <c r="C65" t="s">
+        <v>443</v>
+      </c>
+      <c r="D65" t="s">
+        <v>29</v>
+      </c>
+      <c r="E65" t="s">
         <v>11</v>
       </c>
-      <c r="F43" t="b">
+      <c r="F65" t="b">
         <v>0</v>
       </c>
-      <c r="G43" t="s">
-        <v>31</v>
-      </c>
-      <c r="H43" t="s">
-        <v>506</v>
-      </c>
-      <c r="I43" t="str">
+      <c r="G65" t="s">
+        <v>30</v>
+      </c>
+      <c r="H65" t="s">
+        <v>144</v>
+      </c>
+      <c r="I65" t="str">
         <f t="shared" si="5"/>
         <v>single-input, double-output</v>
       </c>
-      <c r="J43" t="str">
+      <c r="J65" t="str">
         <f t="shared" si="6"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>102</v>
-      </c>
-      <c r="B44" t="s">
-        <v>103</v>
-      </c>
-      <c r="C44" t="s">
-        <v>450</v>
-      </c>
-      <c r="D44" t="s">
-        <v>30</v>
-      </c>
-      <c r="E44" t="s">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>145</v>
+      </c>
+      <c r="B66" t="s">
+        <v>146</v>
+      </c>
+      <c r="C66" t="s">
+        <v>407</v>
+      </c>
+      <c r="D66" t="s">
+        <v>10</v>
+      </c>
+      <c r="E66" t="s">
         <v>11</v>
       </c>
-      <c r="F44" t="b">
+      <c r="F66" t="b">
         <v>1</v>
       </c>
-      <c r="G44" t="s">
-        <v>21</v>
-      </c>
-      <c r="H44" t="b">
-        <v>0</v>
-      </c>
-      <c r="I44" t="str">
+      <c r="G66" t="s">
+        <v>12</v>
+      </c>
+      <c r="H66" t="str">
+        <f>IF(D66="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
+      </c>
+      <c r="I66" t="str">
         <f t="shared" si="5"/>
         <v>single-input, double-output</v>
       </c>
-      <c r="J44" t="str">
+      <c r="J66" t="str">
         <f t="shared" si="6"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>474</v>
-      </c>
-      <c r="B45" t="s">
-        <v>473</v>
-      </c>
-      <c r="C45" t="s">
-        <v>475</v>
-      </c>
-      <c r="D45" t="s">
-        <v>10</v>
-      </c>
-      <c r="E45" t="s">
-        <v>18</v>
-      </c>
-      <c r="F45" t="b">
-        <v>1</v>
-      </c>
-      <c r="G45" t="s">
-        <v>12</v>
-      </c>
-      <c r="H45" t="s">
-        <v>476</v>
-      </c>
-      <c r="I45" t="str">
-        <f t="shared" si="5"/>
-        <v>reactive single-inlet, double-outlet</v>
-      </c>
-      <c r="J45" t="str">
-        <f t="shared" si="6"/>
-        <v>sidor_methods</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>477</v>
-      </c>
-      <c r="B46" t="s">
-        <v>455</v>
-      </c>
-      <c r="C46" t="s">
-        <v>451</v>
-      </c>
-      <c r="D46" t="s">
-        <v>30</v>
-      </c>
-      <c r="E46" t="s">
-        <v>18</v>
-      </c>
-      <c r="F46" t="b">
-        <v>1</v>
-      </c>
-      <c r="G46" t="s">
-        <v>31</v>
-      </c>
-      <c r="H46" t="s">
-        <v>478</v>
-      </c>
-      <c r="I46" t="str">
-        <f t="shared" si="5"/>
-        <v>reactive single-inlet, double-outlet</v>
-      </c>
-      <c r="J46" t="str">
-        <f t="shared" si="6"/>
-        <v>sidor_methods</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>104</v>
-      </c>
-      <c r="B47" t="s">
-        <v>105</v>
-      </c>
-      <c r="C47" t="s">
-        <v>441</v>
-      </c>
-      <c r="D47" t="s">
-        <v>10</v>
-      </c>
-      <c r="E47" t="s">
-        <v>27</v>
-      </c>
-      <c r="F47" t="b">
-        <v>1</v>
-      </c>
-      <c r="G47" t="s">
-        <v>12</v>
-      </c>
-      <c r="H47" t="str">
-        <f>IF(D47="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
-      </c>
-      <c r="I47" t="str">
-        <f t="shared" ref="I47:I92" si="7">IF(E47="SIDO","single-input, double-output",IF(E47="SISO","single-input, single-output",IF(E47="PT","pass-through",IF(E47="DISO","double-input, single-output",IF(E47="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
-        <v>pass-through</v>
-      </c>
-      <c r="J47" t="str">
-        <f t="shared" ref="J47:J92" si="8">IF(E47="SIDO","sido_methods",IF(E47="SISO","siso_methods",IF(E47="PT","pt_methods",IF(E47="DISO","diso_methods",IF(E47="SIDO reactive","sidor_methods","")))))</f>
-        <v>pt_methods</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>106</v>
-      </c>
-      <c r="B48" t="s">
-        <v>107</v>
-      </c>
-      <c r="C48" t="s">
-        <v>440</v>
-      </c>
-      <c r="D48" t="s">
-        <v>10</v>
-      </c>
-      <c r="E48" t="s">
-        <v>27</v>
-      </c>
-      <c r="F48" t="b">
-        <v>1</v>
-      </c>
-      <c r="G48" t="s">
-        <v>12</v>
-      </c>
-      <c r="H48" t="str">
-        <f>IF(D48="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
-      </c>
-      <c r="I48" t="str">
-        <f t="shared" si="7"/>
-        <v>pass-through</v>
-      </c>
-      <c r="J48" t="str">
-        <f t="shared" si="8"/>
-        <v>pt_methods</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>108</v>
-      </c>
-      <c r="B49" t="s">
-        <v>109</v>
-      </c>
-      <c r="C49" t="s">
-        <v>426</v>
-      </c>
-      <c r="D49" t="s">
-        <v>30</v>
-      </c>
-      <c r="E49" t="s">
-        <v>11</v>
-      </c>
-      <c r="F49" t="b">
-        <v>1</v>
-      </c>
-      <c r="G49" t="s">
-        <v>21</v>
-      </c>
-      <c r="H49" t="s">
-        <v>110</v>
-      </c>
-      <c r="I49" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
-      </c>
-      <c r="J49" t="str">
-        <f t="shared" si="8"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>111</v>
-      </c>
-      <c r="B50" t="s">
-        <v>112</v>
-      </c>
-      <c r="C50" t="s">
-        <v>396</v>
-      </c>
-      <c r="D50" t="s">
-        <v>30</v>
-      </c>
-      <c r="E50" t="s">
-        <v>11</v>
-      </c>
-      <c r="F50" t="b">
-        <v>0</v>
-      </c>
-      <c r="G50" t="s">
-        <v>31</v>
-      </c>
-      <c r="H50" t="s">
-        <v>113</v>
-      </c>
-      <c r="I50" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
-      </c>
-      <c r="J50" t="str">
-        <f t="shared" si="8"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>114</v>
-      </c>
-      <c r="B51" t="s">
-        <v>115</v>
-      </c>
-      <c r="C51" t="s">
-        <v>397</v>
-      </c>
-      <c r="D51" t="s">
-        <v>10</v>
-      </c>
-      <c r="E51" t="s">
-        <v>27</v>
-      </c>
-      <c r="F51" t="b">
-        <v>1</v>
-      </c>
-      <c r="G51" t="s">
-        <v>12</v>
-      </c>
-      <c r="H51" t="s">
-        <v>116</v>
-      </c>
-      <c r="I51" t="str">
-        <f t="shared" si="7"/>
-        <v>pass-through</v>
-      </c>
-      <c r="J51" t="str">
-        <f t="shared" si="8"/>
-        <v>pt_methods</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>117</v>
-      </c>
-      <c r="B52" t="s">
-        <v>118</v>
-      </c>
-      <c r="C52" t="s">
-        <v>399</v>
-      </c>
-      <c r="D52" t="s">
-        <v>30</v>
-      </c>
-      <c r="E52" t="s">
-        <v>18</v>
-      </c>
-      <c r="F52" t="b">
-        <v>1</v>
-      </c>
-      <c r="G52" t="s">
-        <v>12</v>
-      </c>
-      <c r="H52" t="s">
-        <v>119</v>
-      </c>
-      <c r="I52" t="str">
-        <f t="shared" si="7"/>
-        <v>reactive single-inlet, double-outlet</v>
-      </c>
-      <c r="J52" t="str">
-        <f t="shared" si="8"/>
-        <v>sidor_methods</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>479</v>
-      </c>
-      <c r="B53" t="s">
-        <v>480</v>
-      </c>
-      <c r="C53" t="s">
-        <v>481</v>
-      </c>
-      <c r="D53" t="s">
-        <v>30</v>
-      </c>
-      <c r="E53" t="s">
-        <v>18</v>
-      </c>
-      <c r="F53" t="b">
-        <v>1</v>
-      </c>
-      <c r="G53" t="s">
-        <v>12</v>
-      </c>
-      <c r="H53" t="s">
-        <v>482</v>
-      </c>
-      <c r="I53" t="str">
-        <f t="shared" si="7"/>
-        <v>reactive single-inlet, double-outlet</v>
-      </c>
-      <c r="J53" t="str">
-        <f t="shared" si="8"/>
-        <v>sidor_methods</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>120</v>
-      </c>
-      <c r="B54" t="s">
-        <v>121</v>
-      </c>
-      <c r="C54" t="s">
-        <v>400</v>
-      </c>
-      <c r="D54" t="s">
-        <v>10</v>
-      </c>
-      <c r="E54" t="s">
-        <v>11</v>
-      </c>
-      <c r="F54" t="b">
-        <v>1</v>
-      </c>
-      <c r="G54" t="s">
-        <v>12</v>
-      </c>
-      <c r="H54" t="str">
-        <f>IF(D54="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
-      </c>
-      <c r="I54" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
-      </c>
-      <c r="J54" t="str">
-        <f t="shared" si="8"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>122</v>
-      </c>
-      <c r="B55" t="s">
-        <v>123</v>
-      </c>
-      <c r="C55" t="s">
-        <v>401</v>
-      </c>
-      <c r="D55" t="s">
-        <v>10</v>
-      </c>
-      <c r="E55" t="s">
-        <v>11</v>
-      </c>
-      <c r="F55" t="b">
-        <v>1</v>
-      </c>
-      <c r="G55" t="s">
-        <v>12</v>
-      </c>
-      <c r="H55" t="str">
-        <f>IF(D55="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
-      </c>
-      <c r="I55" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
-      </c>
-      <c r="J55" t="str">
-        <f t="shared" si="8"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>483</v>
-      </c>
-      <c r="B56" t="s">
-        <v>484</v>
-      </c>
-      <c r="C56" t="s">
-        <v>485</v>
-      </c>
-      <c r="D56" t="s">
-        <v>30</v>
-      </c>
-      <c r="E56" t="s">
-        <v>11</v>
-      </c>
-      <c r="F56" t="b">
-        <v>1</v>
-      </c>
-      <c r="G56" t="s">
-        <v>12</v>
-      </c>
-      <c r="H56" t="s">
-        <v>486</v>
-      </c>
-      <c r="I56" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
-      </c>
-      <c r="J56" t="str">
-        <f t="shared" si="8"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
-        <v>124</v>
-      </c>
-      <c r="B57" t="s">
-        <v>125</v>
-      </c>
-      <c r="C57" t="s">
-        <v>385</v>
-      </c>
-      <c r="D57" t="s">
-        <v>30</v>
-      </c>
-      <c r="E57" t="s">
-        <v>18</v>
-      </c>
-      <c r="F57" t="b">
-        <v>0</v>
-      </c>
-      <c r="G57" t="s">
-        <v>31</v>
-      </c>
-      <c r="H57" t="s">
-        <v>126</v>
-      </c>
-      <c r="I57" t="str">
-        <f t="shared" si="7"/>
-        <v>reactive single-inlet, double-outlet</v>
-      </c>
-      <c r="J57" t="str">
-        <f t="shared" si="8"/>
-        <v>sidor_methods</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
-        <v>487</v>
-      </c>
-      <c r="B58" t="s">
-        <v>488</v>
-      </c>
-      <c r="C58" t="s">
-        <v>489</v>
-      </c>
-      <c r="D58" t="s">
-        <v>30</v>
-      </c>
-      <c r="E58" t="s">
-        <v>18</v>
-      </c>
-      <c r="F58" t="b">
-        <v>1</v>
-      </c>
-      <c r="G58" t="s">
-        <v>12</v>
-      </c>
-      <c r="H58" t="s">
-        <v>490</v>
-      </c>
-      <c r="I58" t="str">
-        <f t="shared" si="7"/>
-        <v>reactive single-inlet, double-outlet</v>
-      </c>
-      <c r="J58" t="str">
-        <f t="shared" si="8"/>
-        <v>sidor_methods</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
-        <v>127</v>
-      </c>
-      <c r="B59" t="s">
-        <v>128</v>
-      </c>
-      <c r="C59" t="s">
-        <v>402</v>
-      </c>
-      <c r="D59" t="s">
-        <v>10</v>
-      </c>
-      <c r="E59" t="s">
-        <v>11</v>
-      </c>
-      <c r="F59" t="b">
-        <v>1</v>
-      </c>
-      <c r="G59" t="s">
-        <v>12</v>
-      </c>
-      <c r="H59" t="str">
-        <f>IF(D59="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
-      </c>
-      <c r="I59" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
-      </c>
-      <c r="J59" t="str">
-        <f t="shared" si="8"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>130</v>
-      </c>
-      <c r="B60" t="s">
-        <v>131</v>
-      </c>
-      <c r="C60" t="s">
-        <v>423</v>
-      </c>
-      <c r="D60" t="s">
-        <v>10</v>
-      </c>
-      <c r="E60" t="s">
-        <v>27</v>
-      </c>
-      <c r="F60" t="b">
-        <v>1</v>
-      </c>
-      <c r="G60" t="s">
-        <v>21</v>
-      </c>
-      <c r="H60" t="s">
-        <v>65</v>
-      </c>
-      <c r="I60" t="str">
-        <f t="shared" si="7"/>
-        <v>pass-through</v>
-      </c>
-      <c r="J60" t="str">
-        <f t="shared" si="8"/>
-        <v>pt_methods</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
-        <v>132</v>
-      </c>
-      <c r="B61" t="s">
-        <v>133</v>
-      </c>
-      <c r="C61" t="s">
-        <v>404</v>
-      </c>
-      <c r="D61" t="s">
-        <v>10</v>
-      </c>
-      <c r="E61" t="s">
-        <v>27</v>
-      </c>
-      <c r="F61" t="b">
-        <v>1</v>
-      </c>
-      <c r="G61" t="s">
-        <v>12</v>
-      </c>
-      <c r="H61" t="str">
-        <f>IF(D61="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
-      </c>
-      <c r="I61" t="str">
-        <f t="shared" si="7"/>
-        <v>pass-through</v>
-      </c>
-      <c r="J61" t="str">
-        <f t="shared" si="8"/>
-        <v>pt_methods</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
-        <v>134</v>
-      </c>
-      <c r="B62" t="s">
-        <v>135</v>
-      </c>
-      <c r="C62" t="s">
-        <v>405</v>
-      </c>
-      <c r="D62" t="s">
-        <v>30</v>
-      </c>
-      <c r="E62" t="s">
-        <v>11</v>
-      </c>
-      <c r="F62" t="b">
-        <v>0</v>
-      </c>
-      <c r="G62" t="s">
-        <v>31</v>
-      </c>
-      <c r="H62" t="s">
-        <v>136</v>
-      </c>
-      <c r="I62" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
-      </c>
-      <c r="J62" t="str">
-        <f t="shared" si="8"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
-        <v>137</v>
-      </c>
-      <c r="B63" t="s">
-        <v>369</v>
-      </c>
-      <c r="C63" t="s">
-        <v>425</v>
-      </c>
-      <c r="D63" t="s">
-        <v>30</v>
-      </c>
-      <c r="E63" t="s">
-        <v>26</v>
-      </c>
-      <c r="F63" t="b">
-        <v>0</v>
-      </c>
-      <c r="G63" t="s">
-        <v>31</v>
-      </c>
-      <c r="H63" t="s">
-        <v>138</v>
-      </c>
-      <c r="I63" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, single-output</v>
-      </c>
-      <c r="J63" t="str">
-        <f t="shared" si="8"/>
-        <v>siso_methods</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
-        <v>139</v>
-      </c>
-      <c r="B64" t="s">
-        <v>140</v>
-      </c>
-      <c r="C64" t="s">
-        <v>424</v>
-      </c>
-      <c r="D64" t="s">
-        <v>30</v>
-      </c>
-      <c r="E64" t="s">
-        <v>26</v>
-      </c>
-      <c r="F64" t="b">
-        <v>0</v>
-      </c>
-      <c r="G64" t="s">
-        <v>31</v>
-      </c>
-      <c r="H64" t="s">
-        <v>141</v>
-      </c>
-      <c r="I64" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, single-output</v>
-      </c>
-      <c r="J64" t="str">
-        <f t="shared" si="8"/>
-        <v>siso_methods</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>491</v>
-      </c>
-      <c r="B65" t="s">
-        <v>492</v>
-      </c>
-      <c r="C65" t="s">
-        <v>493</v>
-      </c>
-      <c r="D65" t="s">
-        <v>30</v>
-      </c>
-      <c r="E65" t="s">
-        <v>18</v>
-      </c>
-      <c r="F65" t="b">
-        <v>1</v>
-      </c>
-      <c r="G65" t="s">
-        <v>12</v>
-      </c>
-      <c r="H65" t="s">
-        <v>494</v>
-      </c>
-      <c r="I65" t="str">
-        <f t="shared" si="7"/>
-        <v>reactive single-inlet, double-outlet</v>
-      </c>
-      <c r="J65" t="str">
-        <f t="shared" si="8"/>
-        <v>sidor_methods</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
-        <v>142</v>
-      </c>
-      <c r="B66" t="s">
-        <v>143</v>
-      </c>
-      <c r="C66" t="s">
-        <v>443</v>
-      </c>
-      <c r="D66" t="s">
-        <v>30</v>
-      </c>
-      <c r="E66" t="s">
-        <v>11</v>
-      </c>
-      <c r="F66" t="b">
-        <v>0</v>
-      </c>
-      <c r="G66" t="s">
-        <v>31</v>
-      </c>
-      <c r="H66" t="s">
-        <v>144</v>
-      </c>
-      <c r="I66" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
-      </c>
-      <c r="J66" t="str">
-        <f t="shared" si="8"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B67" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C67" t="s">
-        <v>407</v>
+        <v>398</v>
       </c>
       <c r="D67" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E67" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F67" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G67" t="s">
-        <v>12</v>
-      </c>
-      <c r="H67" t="str">
-        <f>IF(D67="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>30</v>
+      </c>
+      <c r="H67" t="s">
+        <v>149</v>
       </c>
       <c r="I67" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="5"/>
+        <v>pass-through</v>
       </c>
       <c r="J67" t="str">
-        <f t="shared" si="8"/>
-        <v>sido_methods</v>
+        <f t="shared" si="6"/>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B68" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C68" t="s">
-        <v>398</v>
+        <v>408</v>
       </c>
       <c r="D68" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E68" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F68" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G68" t="s">
-        <v>31</v>
-      </c>
-      <c r="H68" t="s">
-        <v>149</v>
+        <v>12</v>
+      </c>
+      <c r="H68" t="str">
+        <f>IF(D68="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I68" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>pass-through</v>
       </c>
       <c r="J68" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>pt_methods</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B69" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C69" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D69" t="s">
         <v>10</v>
       </c>
       <c r="E69" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F69" t="b">
         <v>1</v>
@@ -4325,26 +4314,26 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I69" t="str">
-        <f t="shared" si="7"/>
-        <v>pass-through</v>
+        <f t="shared" si="5"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J69" t="str">
-        <f t="shared" si="8"/>
-        <v>pt_methods</v>
+        <f t="shared" si="6"/>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B70" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C70" t="s">
-        <v>409</v>
+        <v>447</v>
       </c>
       <c r="D70" t="s">
-        <v>10</v>
+        <v>56</v>
       </c>
       <c r="E70" t="s">
         <v>11</v>
@@ -4355,31 +4344,30 @@
       <c r="G70" t="s">
         <v>12</v>
       </c>
-      <c r="H70" t="str">
-        <f>IF(D70="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H70" t="s">
+        <v>64</v>
       </c>
       <c r="I70" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J70" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B71" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C71" t="s">
-        <v>447</v>
+        <v>410</v>
       </c>
       <c r="D71" t="s">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="E71" t="s">
         <v>11</v>
@@ -4391,29 +4379,29 @@
         <v>12</v>
       </c>
       <c r="H71" t="s">
-        <v>65</v>
+        <v>158</v>
       </c>
       <c r="I71" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J71" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B72" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C72" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D72" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E72" t="s">
         <v>11</v>
@@ -4424,27 +4412,28 @@
       <c r="G72" t="s">
         <v>12</v>
       </c>
-      <c r="H72" t="s">
-        <v>158</v>
+      <c r="H72" t="str">
+        <f>IF(D72="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I72" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J72" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B73" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C73" t="s">
-        <v>411</v>
+        <v>435</v>
       </c>
       <c r="D73" t="s">
         <v>10</v>
@@ -4463,29 +4452,29 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I73" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J73" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B74" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C74" t="s">
-        <v>435</v>
+        <v>412</v>
       </c>
       <c r="D74" t="s">
         <v>10</v>
       </c>
       <c r="E74" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F74" t="b">
         <v>1</v>
@@ -4498,29 +4487,29 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I74" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="5"/>
+        <v>pass-through</v>
       </c>
       <c r="J74" t="str">
-        <f t="shared" si="8"/>
-        <v>sido_methods</v>
+        <f t="shared" si="6"/>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B75" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C75" t="s">
-        <v>412</v>
+        <v>433</v>
       </c>
       <c r="D75" t="s">
         <v>10</v>
       </c>
       <c r="E75" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F75" t="b">
         <v>1</v>
@@ -4533,29 +4522,29 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I75" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>pass-through</v>
       </c>
       <c r="J75" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>pt_methods</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B76" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C76" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="D76" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E76" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F76" t="b">
         <v>1</v>
@@ -4563,34 +4552,33 @@
       <c r="G76" t="s">
         <v>12</v>
       </c>
-      <c r="H76" t="str">
-        <f>IF(D76="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H76" t="s">
+        <v>169</v>
       </c>
       <c r="I76" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>pass-through</v>
       </c>
       <c r="J76" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>pt_methods</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>167</v>
+        <v>495</v>
       </c>
       <c r="B77" t="s">
-        <v>168</v>
+        <v>496</v>
       </c>
       <c r="C77" t="s">
-        <v>430</v>
+        <v>497</v>
       </c>
       <c r="D77" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E77" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F77" t="b">
         <v>1</v>
@@ -4599,32 +4587,32 @@
         <v>12</v>
       </c>
       <c r="H77" t="s">
-        <v>169</v>
+        <v>498</v>
       </c>
       <c r="I77" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>pass-through</v>
       </c>
       <c r="J77" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>pt_methods</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="B78" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="C78" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="D78" t="s">
         <v>10</v>
       </c>
       <c r="E78" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F78" t="b">
         <v>1</v>
@@ -4633,169 +4621,170 @@
         <v>12</v>
       </c>
       <c r="H78" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="I78" t="str">
-        <f t="shared" si="7"/>
-        <v>pass-through</v>
+        <f t="shared" si="5"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J78" t="str">
-        <f t="shared" si="8"/>
-        <v>pt_methods</v>
+        <f t="shared" si="6"/>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="B79" t="s">
-        <v>500</v>
+        <v>456</v>
       </c>
       <c r="C79" t="s">
-        <v>501</v>
+        <v>452</v>
       </c>
       <c r="D79" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E79" t="s">
         <v>11</v>
       </c>
       <c r="F79" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G79" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="H79" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="I79" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J79" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>503</v>
+        <v>170</v>
       </c>
       <c r="B80" t="s">
-        <v>456</v>
+        <v>171</v>
       </c>
       <c r="C80" t="s">
-        <v>452</v>
+        <v>442</v>
       </c>
       <c r="D80" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E80" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F80" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G80" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H80" t="s">
-        <v>504</v>
+        <v>172</v>
       </c>
       <c r="I80" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="5"/>
+        <v>pass-through</v>
       </c>
       <c r="J80" t="str">
-        <f t="shared" si="8"/>
-        <v>sido_methods</v>
+        <f t="shared" si="6"/>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B81" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C81" t="s">
-        <v>442</v>
+        <v>431</v>
       </c>
       <c r="D81" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E81" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F81" t="b">
         <v>1</v>
       </c>
       <c r="G81" t="s">
-        <v>21</v>
-      </c>
-      <c r="H81" t="s">
-        <v>172</v>
+        <v>20</v>
+      </c>
+      <c r="H81" t="str">
+        <f>IF(D81="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I81" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>pass-through</v>
       </c>
       <c r="J81" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>pt_methods</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B82" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C82" t="s">
-        <v>431</v>
+        <v>413</v>
       </c>
       <c r="D82" t="s">
         <v>10</v>
       </c>
       <c r="E82" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F82" t="b">
         <v>1</v>
       </c>
       <c r="G82" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="H82" t="str">
         <f>IF(D82="basic","cost_power_law_flow")</f>
         <v>cost_power_law_flow</v>
       </c>
       <c r="I82" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>pass-through</v>
       </c>
       <c r="J82" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>pt_methods</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B83" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C83" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D83" t="s">
         <v>10</v>
       </c>
       <c r="E83" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F83" t="b">
         <v>1</v>
@@ -4808,23 +4797,23 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I83" t="str">
-        <f t="shared" si="7"/>
-        <v>pass-through</v>
+        <f t="shared" si="5"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J83" t="str">
-        <f t="shared" si="8"/>
-        <v>pt_methods</v>
+        <f t="shared" si="6"/>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B84" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C84" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="D84" t="s">
         <v>10</v>
@@ -4843,29 +4832,29 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I84" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J84" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B85" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C85" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D85" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E85" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F85" t="b">
         <v>1</v>
@@ -4873,34 +4862,33 @@
       <c r="G85" t="s">
         <v>12</v>
       </c>
-      <c r="H85" t="str">
-        <f>IF(D85="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H85" t="s">
+        <v>183</v>
       </c>
       <c r="I85" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="5"/>
+        <v>single-input, single-output</v>
       </c>
       <c r="J85" t="str">
-        <f t="shared" si="8"/>
-        <v>sido_methods</v>
+        <f t="shared" si="6"/>
+        <v>siso_methods</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B86" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C86" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D86" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E86" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F86" t="b">
         <v>1</v>
@@ -4909,32 +4897,32 @@
         <v>12</v>
       </c>
       <c r="H86" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="I86" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>single-input, single-output</v>
       </c>
       <c r="J86" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>siso_methods</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B87" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C87" t="s">
-        <v>417</v>
+        <v>453</v>
       </c>
       <c r="D87" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="E87" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F87" t="b">
         <v>1</v>
@@ -4943,29 +4931,29 @@
         <v>12</v>
       </c>
       <c r="H87" t="s">
-        <v>186</v>
+        <v>460</v>
       </c>
       <c r="I87" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, single-output</v>
+        <f t="shared" si="5"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J87" t="str">
-        <f t="shared" si="8"/>
-        <v>siso_methods</v>
+        <f t="shared" si="6"/>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B88" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C88" t="s">
-        <v>453</v>
+        <v>420</v>
       </c>
       <c r="D88" t="s">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="E88" t="s">
         <v>11</v>
@@ -4976,27 +4964,28 @@
       <c r="G88" t="s">
         <v>12</v>
       </c>
-      <c r="H88" t="s">
-        <v>460</v>
+      <c r="H88" t="str">
+        <f>IF(D88="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I88" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J88" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B89" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C89" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D89" t="s">
         <v>10</v>
@@ -5015,120 +5004,85 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I89" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J89" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>sido_methods</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B90" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C90" t="s">
-        <v>419</v>
+        <v>438</v>
       </c>
       <c r="D90" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E90" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F90" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G90" t="s">
-        <v>12</v>
-      </c>
-      <c r="H90" t="str">
-        <f>IF(D90="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>30</v>
+      </c>
+      <c r="H90" t="s">
+        <v>64</v>
       </c>
       <c r="I90" t="str">
-        <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="5"/>
+        <v>pass-through</v>
       </c>
       <c r="J90" t="str">
-        <f t="shared" si="8"/>
-        <v>sido_methods</v>
+        <f t="shared" si="6"/>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B91" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C91" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D91" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E91" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F91" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G91" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H91" t="s">
-        <v>65</v>
+        <v>197</v>
       </c>
       <c r="I91" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>pass-through</v>
       </c>
       <c r="J91" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
-        <v>195</v>
-      </c>
-      <c r="B92" t="s">
-        <v>196</v>
-      </c>
-      <c r="C92" t="s">
-        <v>439</v>
-      </c>
-      <c r="D92" t="s">
-        <v>30</v>
-      </c>
-      <c r="E92" t="s">
-        <v>27</v>
-      </c>
-      <c r="F92" t="b">
-        <v>1</v>
-      </c>
-      <c r="G92" t="s">
-        <v>21</v>
-      </c>
-      <c r="H92" t="s">
-        <v>197</v>
-      </c>
-      <c r="I92" t="str">
-        <f t="shared" si="7"/>
-        <v>pass-through</v>
-      </c>
-      <c r="J92" t="str">
-        <f t="shared" si="8"/>
-        <v>pt_methods</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J92">
-    <sortCondition ref="B2:B92"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J91">
+    <sortCondition ref="B2:B91"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6189,7 +6143,7 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B56" t="str">
         <f t="shared" si="0"/>
@@ -6629,7 +6583,7 @@
     </row>
     <row r="2" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
         <v>383</v>
@@ -6637,7 +6591,7 @@
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
         <v>421</v>
@@ -6645,7 +6599,7 @@
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
         <v>445</v>
@@ -6661,7 +6615,7 @@
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
         <v>374</v>
@@ -6669,7 +6623,7 @@
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C7" t="s">
         <v>375</v>
@@ -6677,7 +6631,7 @@
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
         <v>384</v>
@@ -6693,7 +6647,7 @@
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
         <v>427</v>
@@ -6701,7 +6655,7 @@
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
         <v>386</v>
@@ -6709,7 +6663,7 @@
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s">
         <v>444</v>
@@ -6717,7 +6671,7 @@
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
         <v>388</v>
@@ -6725,7 +6679,7 @@
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C14" t="s">
         <v>387</v>
@@ -6733,7 +6687,7 @@
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C15" t="s">
         <v>432</v>
@@ -6741,7 +6695,7 @@
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C16" t="s">
         <v>406</v>
@@ -6749,7 +6703,7 @@
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C17" t="s">
         <v>434</v>
@@ -6757,7 +6711,7 @@
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C18" t="s">
         <v>415</v>
@@ -6765,7 +6719,7 @@
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C19" t="s">
         <v>448</v>
@@ -6773,7 +6727,7 @@
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C20" t="s">
         <v>449</v>
@@ -6781,7 +6735,7 @@
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C21" t="s">
         <v>377</v>
@@ -6789,7 +6743,7 @@
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C22" t="s">
         <v>389</v>
@@ -6797,7 +6751,7 @@
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C23" t="s">
         <v>378</v>
@@ -6805,7 +6759,7 @@
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C24" t="s">
         <v>390</v>
@@ -6813,7 +6767,7 @@
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C25" t="s">
         <v>379</v>
@@ -6821,7 +6775,7 @@
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C26" t="s">
         <v>391</v>
@@ -6829,7 +6783,7 @@
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C27" t="s">
         <v>380</v>
@@ -6837,7 +6791,7 @@
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C28" t="s">
         <v>429</v>
@@ -6845,7 +6799,7 @@
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C29" t="s">
         <v>394</v>
@@ -6853,7 +6807,7 @@
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C30" t="s">
         <v>381</v>
@@ -6861,7 +6815,7 @@
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C31" t="s">
         <v>395</v>
@@ -6869,7 +6823,7 @@
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C32" t="s">
         <v>436</v>
@@ -6877,7 +6831,7 @@
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C33" t="s">
         <v>392</v>
@@ -6885,7 +6839,7 @@
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C34" t="s">
         <v>393</v>
@@ -6893,7 +6847,7 @@
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C35" t="s">
         <v>437</v>
@@ -6901,7 +6855,7 @@
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C36" t="s">
         <v>422</v>
@@ -6909,7 +6863,7 @@
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C37" t="s">
         <v>428</v>
@@ -6917,7 +6871,7 @@
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C38" t="s">
         <v>450</v>
@@ -6933,7 +6887,7 @@
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C40" t="s">
         <v>441</v>
@@ -6941,7 +6895,7 @@
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C41" t="s">
         <v>440</v>
@@ -6949,7 +6903,7 @@
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C42" t="s">
         <v>426</v>
@@ -6957,7 +6911,7 @@
     </row>
     <row r="43" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C43" t="s">
         <v>396</v>
@@ -6965,7 +6919,7 @@
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C44" t="s">
         <v>397</v>
@@ -6973,7 +6927,7 @@
     </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C45" t="s">
         <v>399</v>
@@ -6981,7 +6935,7 @@
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C46" t="s">
         <v>400</v>
@@ -6989,7 +6943,7 @@
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C47" t="s">
         <v>401</v>
@@ -6997,7 +6951,7 @@
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C48" t="s">
         <v>385</v>
@@ -7005,7 +6959,7 @@
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C49" t="s">
         <v>402</v>

</xml_diff>